<commit_message>
feat(logging): enable longtable output via injected LongTableWriter
- Add static LongTableWriter in GridModelActor with setLongWriter(...) injection
- Emit RUN meta (project/scenario/hash_tag) exactly once from GMA
- Guard all longtable writes (null-safe) to prevent NPE before injection
3S1T v0.1 baseline: DC longtable stabilised, brake split signals added

- Stabilised 3S1T (3 substations, 1 train) DC scenario as reference baseline
- Added logging for P_brk_req_W, P_brk_net_W and P_brk_res_W per train
- Logged substation V_V, I_A, P_net_W and P_loss_W and line I_A/P_W for verification
- Clarified that Train.I_A and Train.P_net_W are not yet physically valid in v0.1
- Updated README and docs to describe the 3S1T v0.1 baseline and known limitations
</commit_message>
<xml_diff>
--- a/project/3subs1train/T1/A-B.xlsx
+++ b/project/3subs1train/T1/A-B.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tools\dc-simulator\project\3subs1train\T1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6DCF7CF-79E3-4C4E-AB52-2672AEE496DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30BD48A6-E4E7-468A-8CB6-E09DFFED0220}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17025" xr2:uid="{ABD8D7A9-F49A-425C-BE6F-CA7411EF6D88}"/>
   </bookViews>
@@ -2340,79 +2340,79 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>2500</c:v>
+                  <c:v>-2500</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>2400</c:v>
+                  <c:v>-2400</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>2300</c:v>
+                  <c:v>-2300</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>2200</c:v>
+                  <c:v>-2200</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>2100</c:v>
+                  <c:v>-2100</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>2000</c:v>
+                  <c:v>-2000</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>1900</c:v>
+                  <c:v>-1900</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>1800</c:v>
+                  <c:v>-1800</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>1700</c:v>
+                  <c:v>-1700</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>1600</c:v>
+                  <c:v>-1600</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>1500</c:v>
+                  <c:v>-1500</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>1400</c:v>
+                  <c:v>-1400</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>1300</c:v>
+                  <c:v>-1300</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>1200</c:v>
+                  <c:v>-1200</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>1100</c:v>
+                  <c:v>-1100</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>1000</c:v>
+                  <c:v>-1000</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>900</c:v>
+                  <c:v>-900</c:v>
                 </c:pt>
                 <c:pt idx="96">
-                  <c:v>800</c:v>
+                  <c:v>-800</c:v>
                 </c:pt>
                 <c:pt idx="97">
-                  <c:v>700</c:v>
+                  <c:v>-700</c:v>
                 </c:pt>
                 <c:pt idx="98">
-                  <c:v>600</c:v>
+                  <c:v>-600</c:v>
                 </c:pt>
                 <c:pt idx="99">
-                  <c:v>500</c:v>
+                  <c:v>-500</c:v>
                 </c:pt>
                 <c:pt idx="100">
-                  <c:v>400</c:v>
+                  <c:v>-400</c:v>
                 </c:pt>
                 <c:pt idx="101">
-                  <c:v>300</c:v>
+                  <c:v>-300</c:v>
                 </c:pt>
                 <c:pt idx="102">
-                  <c:v>200</c:v>
+                  <c:v>-200</c:v>
                 </c:pt>
                 <c:pt idx="103">
-                  <c:v>100</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="104">
                   <c:v>0</c:v>
@@ -2645,6 +2645,924 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CL"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>speed [m/s]</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$B$2:$B$106</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="105"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>51</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>53</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>54</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>55</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>56</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>57</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>58</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>59</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>61</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>62</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>65</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>66</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>67</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>68</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>69</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>71</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>73</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>74</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>76</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>77</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>78</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>79</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>81</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>82</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>83</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>84</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>86</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>87</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>88</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>89</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>91</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>93</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>94</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>96</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>97</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>98</c:v>
+                </c:pt>
+                <c:pt idx="99">
+                  <c:v>99</c:v>
+                </c:pt>
+                <c:pt idx="100">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="101">
+                  <c:v>101</c:v>
+                </c:pt>
+                <c:pt idx="102">
+                  <c:v>102</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>103</c:v>
+                </c:pt>
+                <c:pt idx="104">
+                  <c:v>104</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$C$2:$C$106</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="105"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="99">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="100">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="101">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="102">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="104">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-0E6E-49AD-9663-0C11717BFD61}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1429082416"/>
+        <c:axId val="1429082896"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1429082416"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1429082896"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1429082896"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1429082416"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-CL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -2725,6 +3643,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -3757,20 +4715,536 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3798,15 +5272,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
+      <xdr:colOff>295275</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3826,6 +5300,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>504825</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F08784E6-550D-DD45-0497-F697BBBB22B0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4196,7 +5706,7 @@
         <v>100</v>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F86" si="2">IF(A3&lt;0,A3*C3*100,0)</f>
+        <f t="shared" ref="F3:F28" si="2">IF(A3&lt;0,A3*C3*100,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5228,7 +6738,7 @@
         <v>0</v>
       </c>
       <c r="F46">
-        <f t="shared" ref="F46:F80" si="9">IF(A46&lt;0,A46*C46*100,0)</f>
+        <f t="shared" ref="F46:F106" si="9">IF(A46&lt;0,A46*C46*100,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -6071,8 +7581,8 @@
         <v>0</v>
       </c>
       <c r="F81">
-        <f>(IF(A81&lt;0,A81*C81*100,0))*-1</f>
-        <v>2500</v>
+        <f t="shared" si="9"/>
+        <v>-2500</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
@@ -6095,8 +7605,8 @@
         <v>0</v>
       </c>
       <c r="F82">
-        <f>(IF(A82&lt;0,A82*C82*100,0))*-1</f>
-        <v>2400</v>
+        <f t="shared" si="9"/>
+        <v>-2400</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
@@ -6119,8 +7629,8 @@
         <v>0</v>
       </c>
       <c r="F83">
-        <f>(IF(A83&lt;0,A83*C83*100,0))*-1</f>
-        <v>2300</v>
+        <f t="shared" si="9"/>
+        <v>-2300</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
@@ -6143,8 +7653,8 @@
         <v>0</v>
       </c>
       <c r="F84">
-        <f>(IF(A84&lt;0,A84*C84*100,0))*-1</f>
-        <v>2200</v>
+        <f t="shared" si="9"/>
+        <v>-2200</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
@@ -6167,8 +7677,8 @@
         <v>0</v>
       </c>
       <c r="F85">
-        <f>(IF(A85&lt;0,A85*C85*100,0))*-1</f>
-        <v>2100</v>
+        <f t="shared" si="9"/>
+        <v>-2100</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
@@ -6191,8 +7701,8 @@
         <v>0</v>
       </c>
       <c r="F86">
-        <f>(IF(A86&lt;0,A86*C86*100,0))*-1</f>
-        <v>2000</v>
+        <f t="shared" si="9"/>
+        <v>-2000</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -6215,8 +7725,8 @@
         <v>0</v>
       </c>
       <c r="F87">
-        <f>(IF(A87&lt;0,A87*C87*100,0))*-1</f>
-        <v>1900</v>
+        <f t="shared" si="9"/>
+        <v>-1900</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
@@ -6239,8 +7749,8 @@
         <v>0</v>
       </c>
       <c r="F88">
-        <f>(IF(A88&lt;0,A88*C88*100,0))*-1</f>
-        <v>1800</v>
+        <f t="shared" si="9"/>
+        <v>-1800</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
@@ -6263,8 +7773,8 @@
         <v>0</v>
       </c>
       <c r="F89">
-        <f>(IF(A89&lt;0,A89*C89*100,0))*-1</f>
-        <v>1700</v>
+        <f t="shared" si="9"/>
+        <v>-1700</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
@@ -6287,8 +7797,8 @@
         <v>0</v>
       </c>
       <c r="F90">
-        <f>(IF(A90&lt;0,A90*C90*100,0))*-1</f>
-        <v>1600</v>
+        <f t="shared" si="9"/>
+        <v>-1600</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
@@ -6311,8 +7821,8 @@
         <v>0</v>
       </c>
       <c r="F91">
-        <f>(IF(A91&lt;0,A91*C91*100,0))*-1</f>
-        <v>1500</v>
+        <f t="shared" si="9"/>
+        <v>-1500</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
@@ -6335,8 +7845,8 @@
         <v>0</v>
       </c>
       <c r="F92">
-        <f>(IF(A92&lt;0,A92*C92*100,0))*-1</f>
-        <v>1400</v>
+        <f t="shared" si="9"/>
+        <v>-1400</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -6359,8 +7869,8 @@
         <v>0</v>
       </c>
       <c r="F93">
-        <f>(IF(A93&lt;0,A93*C93*100,0))*-1</f>
-        <v>1300</v>
+        <f t="shared" si="9"/>
+        <v>-1300</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
@@ -6383,8 +7893,8 @@
         <v>0</v>
       </c>
       <c r="F94">
-        <f>(IF(A94&lt;0,A94*C94*100,0))*-1</f>
-        <v>1200</v>
+        <f t="shared" si="9"/>
+        <v>-1200</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
@@ -6407,8 +7917,8 @@
         <v>0</v>
       </c>
       <c r="F95">
-        <f>(IF(A95&lt;0,A95*C95*100,0))*-1</f>
-        <v>1100</v>
+        <f t="shared" si="9"/>
+        <v>-1100</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
@@ -6431,8 +7941,8 @@
         <v>0</v>
       </c>
       <c r="F96">
-        <f>(IF(A96&lt;0,A96*C96*100,0))*-1</f>
-        <v>1000</v>
+        <f t="shared" si="9"/>
+        <v>-1000</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
@@ -6455,8 +7965,8 @@
         <v>0</v>
       </c>
       <c r="F97">
-        <f>(IF(A97&lt;0,A97*C97*100,0))*-1</f>
-        <v>900</v>
+        <f t="shared" si="9"/>
+        <v>-900</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
@@ -6479,8 +7989,8 @@
         <v>0</v>
       </c>
       <c r="F98">
-        <f>(IF(A98&lt;0,A98*C98*100,0))*-1</f>
-        <v>800</v>
+        <f t="shared" si="9"/>
+        <v>-800</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
@@ -6503,8 +8013,8 @@
         <v>0</v>
       </c>
       <c r="F99">
-        <f>(IF(A99&lt;0,A99*C99*100,0))*-1</f>
-        <v>700</v>
+        <f t="shared" si="9"/>
+        <v>-700</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
@@ -6527,8 +8037,8 @@
         <v>0</v>
       </c>
       <c r="F100">
-        <f>(IF(A100&lt;0,A100*C100*100,0))*-1</f>
-        <v>600</v>
+        <f t="shared" si="9"/>
+        <v>-600</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
@@ -6551,8 +8061,8 @@
         <v>0</v>
       </c>
       <c r="F101">
-        <f>(IF(A101&lt;0,A101*C101*100,0))*-1</f>
-        <v>500</v>
+        <f t="shared" si="9"/>
+        <v>-500</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -6575,8 +8085,8 @@
         <v>0</v>
       </c>
       <c r="F102">
-        <f>(IF(A102&lt;0,A102*C102*100,0))*-1</f>
-        <v>400</v>
+        <f t="shared" si="9"/>
+        <v>-400</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
@@ -6599,8 +8109,8 @@
         <v>0</v>
       </c>
       <c r="F103">
-        <f>(IF(A103&lt;0,A103*C103*100,0))*-1</f>
-        <v>300</v>
+        <f t="shared" si="9"/>
+        <v>-300</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
@@ -6623,8 +8133,8 @@
         <v>0</v>
       </c>
       <c r="F104">
-        <f>(IF(A104&lt;0,A104*C104*100,0))*-1</f>
-        <v>200</v>
+        <f t="shared" si="9"/>
+        <v>-200</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
@@ -6647,8 +8157,8 @@
         <v>0</v>
       </c>
       <c r="F105">
-        <f>(IF(A105&lt;0,A105*C105*100,0))*-1</f>
-        <v>100</v>
+        <f t="shared" si="9"/>
+        <v>-100</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
@@ -6671,7 +8181,7 @@
         <v>0</v>
       </c>
       <c r="F106">
-        <f>(IF(A106&lt;0,A106*C106*100,0))*-1</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
test(v0.8): add minitests guarding dynamic topology, substation coupling and train voltage logging
- Guard against hardcoded train node indices in solver
- Ensure NetBuilder includes substations and trains when dynamic lines are enabled
- Verify Train.V_V is logged when TrainData exists
- Kill legacy probe-induced false zero-voltage failures
</commit_message>
<xml_diff>
--- a/project/3subs1train/T1/A-B.xlsx
+++ b/project/3subs1train/T1/A-B.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tools\dc-simulator\project\3subs1train\T1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30BD48A6-E4E7-468A-8CB6-E09DFFED0220}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C323FE4E-99F0-4E59-9E20-E32067580597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17025" xr2:uid="{ABD8D7A9-F49A-425C-BE6F-CA7411EF6D88}"/>
   </bookViews>
@@ -504,319 +504,319 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="105"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>3100</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.0000000000000001E-4</c:v>
+                  <c:v>3100.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2E-3</c:v>
+                  <c:v>3102</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.4999999999999997E-3</c:v>
+                  <c:v>3104.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.0000000000000002E-3</c:v>
+                  <c:v>3108</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.2500000000000001E-2</c:v>
+                  <c:v>3112.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.7999999999999999E-2</c:v>
+                  <c:v>3118</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.4500000000000001E-2</c:v>
+                  <c:v>3124.5</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.2000000000000001E-2</c:v>
+                  <c:v>3132</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4.0500000000000001E-2</c:v>
+                  <c:v>3140.5</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.05</c:v>
+                  <c:v>3150</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>6.0499999999999998E-2</c:v>
+                  <c:v>3160.5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>7.1999999999999995E-2</c:v>
+                  <c:v>3172</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>8.4500000000000006E-2</c:v>
+                  <c:v>3184.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>9.8000000000000004E-2</c:v>
+                  <c:v>3198</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.1125</c:v>
+                  <c:v>3212.5</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.128</c:v>
+                  <c:v>3228</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.14449999999999999</c:v>
+                  <c:v>3244.5</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.16200000000000001</c:v>
+                  <c:v>3262</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.18049999999999999</c:v>
+                  <c:v>3280.5</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.2</c:v>
+                  <c:v>3300</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.2205</c:v>
+                  <c:v>3320.5</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.24199999999999999</c:v>
+                  <c:v>3342</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.26450000000000001</c:v>
+                  <c:v>3364.5</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.28799999999999998</c:v>
+                  <c:v>3388</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.3125</c:v>
+                  <c:v>3412.5</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.33750000000000002</c:v>
+                  <c:v>3437.5</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.36249999999999999</c:v>
+                  <c:v>3462.5</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.38750000000000001</c:v>
+                  <c:v>3487.5</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.41249999999999998</c:v>
+                  <c:v>3512.5</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.4375</c:v>
+                  <c:v>3537.5</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.46250000000000002</c:v>
+                  <c:v>3562.5</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.48749999999999999</c:v>
+                  <c:v>3587.5</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.51249999999999996</c:v>
+                  <c:v>3612.5</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>0.53749999999999998</c:v>
+                  <c:v>3637.5</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>0.5625</c:v>
+                  <c:v>3662.5</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>0.58750000000000002</c:v>
+                  <c:v>3687.5</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>0.61250000000000004</c:v>
+                  <c:v>3712.5</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>0.63749999999999996</c:v>
+                  <c:v>3737.5</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>0.66249999999999998</c:v>
+                  <c:v>3762.5</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>0.6875</c:v>
+                  <c:v>3787.5</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>0.71250000000000002</c:v>
+                  <c:v>3812.5</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>0.73750000000000004</c:v>
+                  <c:v>3837.5</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>0.76249999999999996</c:v>
+                  <c:v>3862.5</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>0.78749999999999998</c:v>
+                  <c:v>3887.5</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>0.8125</c:v>
+                  <c:v>3912.5</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>0.83750000000000002</c:v>
+                  <c:v>3937.5</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>0.86250000000000004</c:v>
+                  <c:v>3962.5</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>0.88749999999999996</c:v>
+                  <c:v>3987.5</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>0.91249999999999998</c:v>
+                  <c:v>4012.5</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>0.9375</c:v>
+                  <c:v>4037.5</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>0.96250000000000002</c:v>
+                  <c:v>4062.5</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>0.98750000000000004</c:v>
+                  <c:v>4087.5</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>1.0125</c:v>
+                  <c:v>4112.5</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>1.0375000000000001</c:v>
+                  <c:v>4137.5</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>1.0625</c:v>
+                  <c:v>4162.5</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>1.0874999999999999</c:v>
+                  <c:v>4187.5</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>1.1125</c:v>
+                  <c:v>4212.5</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>1.1375</c:v>
+                  <c:v>4237.5</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>1.1625000000000001</c:v>
+                  <c:v>4262.5</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>1.1875</c:v>
+                  <c:v>4287.5</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>1.2124999999999999</c:v>
+                  <c:v>4312.5</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>1.2375</c:v>
+                  <c:v>4337.5</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>1.2625</c:v>
+                  <c:v>4362.5</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>1.2875000000000001</c:v>
+                  <c:v>4387.5</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>1.3125</c:v>
+                  <c:v>4412.5</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>1.3374999999999999</c:v>
+                  <c:v>4437.5</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>1.3625</c:v>
+                  <c:v>4462.5</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>1.3875</c:v>
+                  <c:v>4487.5</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>1.4125000000000001</c:v>
+                  <c:v>4512.5</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>1.4375</c:v>
+                  <c:v>4537.5</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>1.4624999999999999</c:v>
+                  <c:v>4562.5</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>1.4875</c:v>
+                  <c:v>4587.5</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>1.5125</c:v>
+                  <c:v>4612.5</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>1.5375000000000001</c:v>
+                  <c:v>4637.5</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>1.5625</c:v>
+                  <c:v>4662.5</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>1.5874999999999999</c:v>
+                  <c:v>4687.5</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>1.6125</c:v>
+                  <c:v>4712.5</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>1.6375</c:v>
+                  <c:v>4737.5</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>1.6625000000000001</c:v>
+                  <c:v>4762.5</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>1.6870000000000001</c:v>
+                  <c:v>4787</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>1.7104999999999999</c:v>
+                  <c:v>4810.5</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>1.7330000000000001</c:v>
+                  <c:v>4833</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>1.7544999999999999</c:v>
+                  <c:v>4854.5</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>1.7749999999999999</c:v>
+                  <c:v>4875</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>1.7945</c:v>
+                  <c:v>4894.5</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>1.8129999999999999</c:v>
+                  <c:v>4913</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>1.8305</c:v>
+                  <c:v>4930.5</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>1.847</c:v>
+                  <c:v>4947</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>1.8625</c:v>
+                  <c:v>4962.5</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>1.877</c:v>
+                  <c:v>4977</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>1.8905000000000001</c:v>
+                  <c:v>4990.5</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>1.903</c:v>
+                  <c:v>5003</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>1.9145000000000001</c:v>
+                  <c:v>5014.5</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>1.925</c:v>
+                  <c:v>5025</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>1.9345000000000001</c:v>
+                  <c:v>5034.5</c:v>
                 </c:pt>
                 <c:pt idx="96">
-                  <c:v>1.9430000000000001</c:v>
+                  <c:v>5043</c:v>
                 </c:pt>
                 <c:pt idx="97">
-                  <c:v>1.9504999999999999</c:v>
+                  <c:v>5050.5</c:v>
                 </c:pt>
                 <c:pt idx="98">
-                  <c:v>1.9570000000000001</c:v>
+                  <c:v>5057</c:v>
                 </c:pt>
                 <c:pt idx="99">
-                  <c:v>1.9624999999999999</c:v>
+                  <c:v>5062.5</c:v>
                 </c:pt>
                 <c:pt idx="100">
-                  <c:v>1.9670000000000001</c:v>
+                  <c:v>5067</c:v>
                 </c:pt>
                 <c:pt idx="101">
-                  <c:v>1.9704999999999999</c:v>
+                  <c:v>5070.5</c:v>
                 </c:pt>
                 <c:pt idx="102">
-                  <c:v>1.9730000000000001</c:v>
+                  <c:v>5073</c:v>
                 </c:pt>
                 <c:pt idx="103">
-                  <c:v>1.9744999999999999</c:v>
+                  <c:v>5074.5</c:v>
                 </c:pt>
                 <c:pt idx="104">
-                  <c:v>1.9750000000000001</c:v>
+                  <c:v>5075</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5641,10 +5641,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52F5F2CC-9C60-4798-9786-EA69E6C5E2FD}">
-  <dimension ref="A1:I106"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -5664,7 +5664,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -5675,7 +5675,7 @@
         <v>0</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>3100</v>
       </c>
       <c r="E2">
         <f>IF(A2&gt;0,A2*C2*100,0)</f>
@@ -5685,8 +5685,11 @@
         <f>IF(A2&lt;0,A2*C2*100,0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L2">
+        <v>3100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -5698,8 +5701,8 @@
         <v>1</v>
       </c>
       <c r="D3">
-        <f>(D2*1000+C2+0.5*A2)/1000</f>
-        <v>5.0000000000000001E-4</v>
+        <f>(D2+C2+0.5*A2)</f>
+        <v>3100.5</v>
       </c>
       <c r="E3">
         <f t="shared" ref="E3:E86" si="1">IF(A3&gt;0,A3*C3*100,0)</f>
@@ -5710,7 +5713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -5722,8 +5725,8 @@
         <v>2</v>
       </c>
       <c r="D4">
-        <f t="shared" ref="D4:D67" si="3">(D3*1000+C3+0.5*A3)/1000</f>
-        <v>2E-3</v>
+        <f t="shared" ref="D4:D67" si="3">(D3+C3+0.5*A3)</f>
+        <v>3102</v>
       </c>
       <c r="E4">
         <f t="shared" si="1"/>
@@ -5734,7 +5737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -5747,7 +5750,7 @@
       </c>
       <c r="D5">
         <f t="shared" si="3"/>
-        <v>4.4999999999999997E-3</v>
+        <v>3104.5</v>
       </c>
       <c r="E5">
         <f t="shared" si="1"/>
@@ -5758,7 +5761,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
@@ -5771,7 +5774,7 @@
       </c>
       <c r="D6">
         <f t="shared" si="3"/>
-        <v>8.0000000000000002E-3</v>
+        <v>3108</v>
       </c>
       <c r="E6">
         <f t="shared" si="1"/>
@@ -5782,7 +5785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -5795,7 +5798,7 @@
       </c>
       <c r="D7">
         <f t="shared" si="3"/>
-        <v>1.2500000000000001E-2</v>
+        <v>3112.5</v>
       </c>
       <c r="E7">
         <f t="shared" si="1"/>
@@ -5806,7 +5809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
@@ -5819,7 +5822,7 @@
       </c>
       <c r="D8">
         <f t="shared" si="3"/>
-        <v>1.7999999999999999E-2</v>
+        <v>3118</v>
       </c>
       <c r="E8">
         <f t="shared" si="1"/>
@@ -5830,7 +5833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
@@ -5843,7 +5846,7 @@
       </c>
       <c r="D9">
         <f t="shared" si="3"/>
-        <v>2.4500000000000001E-2</v>
+        <v>3124.5</v>
       </c>
       <c r="E9">
         <f t="shared" si="1"/>
@@ -5854,7 +5857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1</v>
       </c>
@@ -5867,7 +5870,7 @@
       </c>
       <c r="D10">
         <f t="shared" si="3"/>
-        <v>3.2000000000000001E-2</v>
+        <v>3132</v>
       </c>
       <c r="E10">
         <f t="shared" si="1"/>
@@ -5878,7 +5881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1</v>
       </c>
@@ -5891,7 +5894,7 @@
       </c>
       <c r="D11">
         <f t="shared" si="3"/>
-        <v>4.0500000000000001E-2</v>
+        <v>3140.5</v>
       </c>
       <c r="E11">
         <f t="shared" si="1"/>
@@ -5902,7 +5905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1</v>
       </c>
@@ -5915,7 +5918,7 @@
       </c>
       <c r="D12">
         <f t="shared" si="3"/>
-        <v>0.05</v>
+        <v>3150</v>
       </c>
       <c r="E12">
         <f t="shared" si="1"/>
@@ -5926,7 +5929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1</v>
       </c>
@@ -5939,7 +5942,7 @@
       </c>
       <c r="D13">
         <f t="shared" si="3"/>
-        <v>6.0499999999999998E-2</v>
+        <v>3160.5</v>
       </c>
       <c r="E13">
         <f t="shared" si="1"/>
@@ -5950,7 +5953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1</v>
       </c>
@@ -5963,7 +5966,7 @@
       </c>
       <c r="D14">
         <f t="shared" si="3"/>
-        <v>7.1999999999999995E-2</v>
+        <v>3172</v>
       </c>
       <c r="E14">
         <f t="shared" si="1"/>
@@ -5974,7 +5977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>1</v>
       </c>
@@ -5987,7 +5990,7 @@
       </c>
       <c r="D15">
         <f t="shared" si="3"/>
-        <v>8.4500000000000006E-2</v>
+        <v>3184.5</v>
       </c>
       <c r="E15">
         <f t="shared" si="1"/>
@@ -5998,7 +6001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1</v>
       </c>
@@ -6011,7 +6014,7 @@
       </c>
       <c r="D16">
         <f t="shared" si="3"/>
-        <v>9.8000000000000004E-2</v>
+        <v>3198</v>
       </c>
       <c r="E16">
         <f t="shared" si="1"/>
@@ -6035,7 +6038,7 @@
       </c>
       <c r="D17">
         <f t="shared" si="3"/>
-        <v>0.1125</v>
+        <v>3212.5</v>
       </c>
       <c r="E17">
         <f t="shared" si="1"/>
@@ -6059,7 +6062,7 @@
       </c>
       <c r="D18">
         <f t="shared" si="3"/>
-        <v>0.128</v>
+        <v>3228</v>
       </c>
       <c r="E18">
         <f t="shared" si="1"/>
@@ -6083,7 +6086,7 @@
       </c>
       <c r="D19">
         <f t="shared" si="3"/>
-        <v>0.14449999999999999</v>
+        <v>3244.5</v>
       </c>
       <c r="E19">
         <f t="shared" si="1"/>
@@ -6107,7 +6110,7 @@
       </c>
       <c r="D20">
         <f t="shared" si="3"/>
-        <v>0.16200000000000001</v>
+        <v>3262</v>
       </c>
       <c r="E20">
         <f t="shared" si="1"/>
@@ -6131,7 +6134,7 @@
       </c>
       <c r="D21">
         <f t="shared" si="3"/>
-        <v>0.18049999999999999</v>
+        <v>3280.5</v>
       </c>
       <c r="E21">
         <f t="shared" si="1"/>
@@ -6155,7 +6158,7 @@
       </c>
       <c r="D22">
         <f t="shared" si="3"/>
-        <v>0.2</v>
+        <v>3300</v>
       </c>
       <c r="E22">
         <f t="shared" si="1"/>
@@ -6179,7 +6182,7 @@
       </c>
       <c r="D23">
         <f t="shared" si="3"/>
-        <v>0.2205</v>
+        <v>3320.5</v>
       </c>
       <c r="E23">
         <f t="shared" si="1"/>
@@ -6203,7 +6206,7 @@
       </c>
       <c r="D24">
         <f t="shared" si="3"/>
-        <v>0.24199999999999999</v>
+        <v>3342</v>
       </c>
       <c r="E24">
         <f t="shared" si="1"/>
@@ -6227,7 +6230,7 @@
       </c>
       <c r="D25">
         <f t="shared" si="3"/>
-        <v>0.26450000000000001</v>
+        <v>3364.5</v>
       </c>
       <c r="E25">
         <f t="shared" si="1"/>
@@ -6251,7 +6254,7 @@
       </c>
       <c r="D26">
         <f t="shared" si="3"/>
-        <v>0.28799999999999998</v>
+        <v>3388</v>
       </c>
       <c r="E26">
         <f t="shared" si="1"/>
@@ -6275,7 +6278,7 @@
       </c>
       <c r="D27">
         <f t="shared" si="3"/>
-        <v>0.3125</v>
+        <v>3412.5</v>
       </c>
       <c r="E27">
         <f t="shared" si="1"/>
@@ -6299,7 +6302,7 @@
       </c>
       <c r="D28">
         <f t="shared" si="3"/>
-        <v>0.33750000000000002</v>
+        <v>3437.5</v>
       </c>
       <c r="E28">
         <f t="shared" si="1"/>
@@ -6323,7 +6326,7 @@
       </c>
       <c r="D29">
         <f t="shared" si="3"/>
-        <v>0.36249999999999999</v>
+        <v>3462.5</v>
       </c>
       <c r="E29">
         <f t="shared" ref="E29:E45" si="5">IF(A29&gt;0,A29*C29*100,0)</f>
@@ -6347,7 +6350,7 @@
       </c>
       <c r="D30">
         <f t="shared" si="3"/>
-        <v>0.38750000000000001</v>
+        <v>3487.5</v>
       </c>
       <c r="E30">
         <f t="shared" si="5"/>
@@ -6371,7 +6374,7 @@
       </c>
       <c r="D31">
         <f t="shared" si="3"/>
-        <v>0.41249999999999998</v>
+        <v>3512.5</v>
       </c>
       <c r="E31">
         <f t="shared" si="5"/>
@@ -6395,7 +6398,7 @@
       </c>
       <c r="D32">
         <f t="shared" si="3"/>
-        <v>0.4375</v>
+        <v>3537.5</v>
       </c>
       <c r="E32">
         <f t="shared" si="5"/>
@@ -6419,7 +6422,7 @@
       </c>
       <c r="D33">
         <f t="shared" si="3"/>
-        <v>0.46250000000000002</v>
+        <v>3562.5</v>
       </c>
       <c r="E33">
         <f t="shared" si="5"/>
@@ -6443,7 +6446,7 @@
       </c>
       <c r="D34">
         <f t="shared" si="3"/>
-        <v>0.48749999999999999</v>
+        <v>3587.5</v>
       </c>
       <c r="E34">
         <f t="shared" si="5"/>
@@ -6467,7 +6470,7 @@
       </c>
       <c r="D35">
         <f t="shared" si="3"/>
-        <v>0.51249999999999996</v>
+        <v>3612.5</v>
       </c>
       <c r="E35">
         <f t="shared" si="5"/>
@@ -6491,7 +6494,7 @@
       </c>
       <c r="D36">
         <f t="shared" si="3"/>
-        <v>0.53749999999999998</v>
+        <v>3637.5</v>
       </c>
       <c r="E36">
         <f t="shared" si="5"/>
@@ -6515,7 +6518,7 @@
       </c>
       <c r="D37">
         <f t="shared" si="3"/>
-        <v>0.5625</v>
+        <v>3662.5</v>
       </c>
       <c r="E37">
         <f t="shared" si="5"/>
@@ -6539,7 +6542,7 @@
       </c>
       <c r="D38">
         <f t="shared" si="3"/>
-        <v>0.58750000000000002</v>
+        <v>3687.5</v>
       </c>
       <c r="E38">
         <f t="shared" si="5"/>
@@ -6563,7 +6566,7 @@
       </c>
       <c r="D39">
         <f t="shared" si="3"/>
-        <v>0.61250000000000004</v>
+        <v>3712.5</v>
       </c>
       <c r="E39">
         <f t="shared" si="5"/>
@@ -6587,7 +6590,7 @@
       </c>
       <c r="D40">
         <f t="shared" si="3"/>
-        <v>0.63749999999999996</v>
+        <v>3737.5</v>
       </c>
       <c r="E40">
         <f t="shared" si="5"/>
@@ -6611,7 +6614,7 @@
       </c>
       <c r="D41">
         <f t="shared" si="3"/>
-        <v>0.66249999999999998</v>
+        <v>3762.5</v>
       </c>
       <c r="E41">
         <f t="shared" si="5"/>
@@ -6635,7 +6638,7 @@
       </c>
       <c r="D42">
         <f t="shared" si="3"/>
-        <v>0.6875</v>
+        <v>3787.5</v>
       </c>
       <c r="E42">
         <f t="shared" si="5"/>
@@ -6659,7 +6662,7 @@
       </c>
       <c r="D43">
         <f t="shared" si="3"/>
-        <v>0.71250000000000002</v>
+        <v>3812.5</v>
       </c>
       <c r="E43">
         <f t="shared" si="5"/>
@@ -6683,7 +6686,7 @@
       </c>
       <c r="D44">
         <f t="shared" si="3"/>
-        <v>0.73750000000000004</v>
+        <v>3837.5</v>
       </c>
       <c r="E44">
         <f t="shared" si="5"/>
@@ -6707,7 +6710,7 @@
       </c>
       <c r="D45">
         <f t="shared" si="3"/>
-        <v>0.76249999999999996</v>
+        <v>3862.5</v>
       </c>
       <c r="E45">
         <f t="shared" si="5"/>
@@ -6731,7 +6734,7 @@
       </c>
       <c r="D46">
         <f t="shared" si="3"/>
-        <v>0.78749999999999998</v>
+        <v>3887.5</v>
       </c>
       <c r="E46">
         <f t="shared" ref="E46:E80" si="8">IF(A46&gt;0,A46*C46*100,0)</f>
@@ -6755,7 +6758,7 @@
       </c>
       <c r="D47">
         <f t="shared" si="3"/>
-        <v>0.8125</v>
+        <v>3912.5</v>
       </c>
       <c r="E47">
         <f t="shared" si="8"/>
@@ -6779,7 +6782,7 @@
       </c>
       <c r="D48">
         <f t="shared" si="3"/>
-        <v>0.83750000000000002</v>
+        <v>3937.5</v>
       </c>
       <c r="E48">
         <f t="shared" si="8"/>
@@ -6803,7 +6806,7 @@
       </c>
       <c r="D49">
         <f t="shared" si="3"/>
-        <v>0.86250000000000004</v>
+        <v>3962.5</v>
       </c>
       <c r="E49">
         <f t="shared" si="8"/>
@@ -6827,7 +6830,7 @@
       </c>
       <c r="D50">
         <f t="shared" si="3"/>
-        <v>0.88749999999999996</v>
+        <v>3987.5</v>
       </c>
       <c r="E50">
         <f t="shared" si="8"/>
@@ -6851,7 +6854,7 @@
       </c>
       <c r="D51">
         <f t="shared" si="3"/>
-        <v>0.91249999999999998</v>
+        <v>4012.5</v>
       </c>
       <c r="E51">
         <f t="shared" si="8"/>
@@ -6875,7 +6878,7 @@
       </c>
       <c r="D52">
         <f t="shared" si="3"/>
-        <v>0.9375</v>
+        <v>4037.5</v>
       </c>
       <c r="E52">
         <f t="shared" si="8"/>
@@ -6899,7 +6902,7 @@
       </c>
       <c r="D53">
         <f t="shared" si="3"/>
-        <v>0.96250000000000002</v>
+        <v>4062.5</v>
       </c>
       <c r="E53">
         <f t="shared" si="8"/>
@@ -6923,7 +6926,7 @@
       </c>
       <c r="D54">
         <f t="shared" si="3"/>
-        <v>0.98750000000000004</v>
+        <v>4087.5</v>
       </c>
       <c r="E54">
         <f t="shared" si="8"/>
@@ -6947,7 +6950,7 @@
       </c>
       <c r="D55">
         <f t="shared" si="3"/>
-        <v>1.0125</v>
+        <v>4112.5</v>
       </c>
       <c r="E55">
         <f t="shared" si="8"/>
@@ -6971,7 +6974,7 @@
       </c>
       <c r="D56">
         <f t="shared" si="3"/>
-        <v>1.0375000000000001</v>
+        <v>4137.5</v>
       </c>
       <c r="E56">
         <f t="shared" si="8"/>
@@ -6995,7 +6998,7 @@
       </c>
       <c r="D57">
         <f t="shared" si="3"/>
-        <v>1.0625</v>
+        <v>4162.5</v>
       </c>
       <c r="E57">
         <f t="shared" si="8"/>
@@ -7019,7 +7022,7 @@
       </c>
       <c r="D58">
         <f t="shared" si="3"/>
-        <v>1.0874999999999999</v>
+        <v>4187.5</v>
       </c>
       <c r="E58">
         <f t="shared" si="8"/>
@@ -7043,7 +7046,7 @@
       </c>
       <c r="D59">
         <f t="shared" si="3"/>
-        <v>1.1125</v>
+        <v>4212.5</v>
       </c>
       <c r="E59">
         <f t="shared" si="8"/>
@@ -7067,7 +7070,7 @@
       </c>
       <c r="D60">
         <f t="shared" si="3"/>
-        <v>1.1375</v>
+        <v>4237.5</v>
       </c>
       <c r="E60">
         <f t="shared" si="8"/>
@@ -7091,7 +7094,7 @@
       </c>
       <c r="D61">
         <f t="shared" si="3"/>
-        <v>1.1625000000000001</v>
+        <v>4262.5</v>
       </c>
       <c r="E61">
         <f t="shared" si="8"/>
@@ -7115,7 +7118,7 @@
       </c>
       <c r="D62">
         <f t="shared" si="3"/>
-        <v>1.1875</v>
+        <v>4287.5</v>
       </c>
       <c r="E62">
         <f t="shared" si="8"/>
@@ -7139,7 +7142,7 @@
       </c>
       <c r="D63">
         <f t="shared" si="3"/>
-        <v>1.2124999999999999</v>
+        <v>4312.5</v>
       </c>
       <c r="E63">
         <f t="shared" si="8"/>
@@ -7163,7 +7166,7 @@
       </c>
       <c r="D64">
         <f t="shared" si="3"/>
-        <v>1.2375</v>
+        <v>4337.5</v>
       </c>
       <c r="E64">
         <f t="shared" si="8"/>
@@ -7187,7 +7190,7 @@
       </c>
       <c r="D65">
         <f t="shared" si="3"/>
-        <v>1.2625</v>
+        <v>4362.5</v>
       </c>
       <c r="E65">
         <f t="shared" si="8"/>
@@ -7211,7 +7214,7 @@
       </c>
       <c r="D66">
         <f t="shared" si="3"/>
-        <v>1.2875000000000001</v>
+        <v>4387.5</v>
       </c>
       <c r="E66">
         <f t="shared" ref="E66:E68" si="11">IF(A66&gt;0,A66*C66*100,0)</f>
@@ -7235,7 +7238,7 @@
       </c>
       <c r="D67">
         <f t="shared" si="3"/>
-        <v>1.3125</v>
+        <v>4412.5</v>
       </c>
       <c r="E67">
         <f t="shared" si="11"/>
@@ -7258,8 +7261,8 @@
         <v>25</v>
       </c>
       <c r="D68">
-        <f t="shared" ref="D68:D106" si="13">(D67*1000+C67+0.5*A67)/1000</f>
-        <v>1.3374999999999999</v>
+        <f t="shared" ref="D68:D106" si="13">(D67+C67+0.5*A67)</f>
+        <v>4437.5</v>
       </c>
       <c r="E68">
         <f t="shared" si="11"/>
@@ -7283,7 +7286,7 @@
       </c>
       <c r="D69">
         <f t="shared" si="13"/>
-        <v>1.3625</v>
+        <v>4462.5</v>
       </c>
       <c r="E69">
         <f t="shared" ref="E69:E71" si="15">IF(A69&gt;0,A69*C69*100,0)</f>
@@ -7307,7 +7310,7 @@
       </c>
       <c r="D70">
         <f t="shared" si="13"/>
-        <v>1.3875</v>
+        <v>4487.5</v>
       </c>
       <c r="E70">
         <f t="shared" si="15"/>
@@ -7331,7 +7334,7 @@
       </c>
       <c r="D71">
         <f t="shared" si="13"/>
-        <v>1.4125000000000001</v>
+        <v>4512.5</v>
       </c>
       <c r="E71">
         <f t="shared" si="15"/>
@@ -7355,7 +7358,7 @@
       </c>
       <c r="D72">
         <f t="shared" si="13"/>
-        <v>1.4375</v>
+        <v>4537.5</v>
       </c>
       <c r="E72">
         <f t="shared" si="8"/>
@@ -7379,7 +7382,7 @@
       </c>
       <c r="D73">
         <f t="shared" si="13"/>
-        <v>1.4624999999999999</v>
+        <v>4562.5</v>
       </c>
       <c r="E73">
         <f t="shared" si="8"/>
@@ -7403,7 +7406,7 @@
       </c>
       <c r="D74">
         <f t="shared" si="13"/>
-        <v>1.4875</v>
+        <v>4587.5</v>
       </c>
       <c r="E74">
         <f t="shared" si="8"/>
@@ -7430,7 +7433,7 @@
       </c>
       <c r="D75">
         <f t="shared" si="13"/>
-        <v>1.5125</v>
+        <v>4612.5</v>
       </c>
       <c r="E75">
         <f t="shared" si="8"/>
@@ -7454,7 +7457,7 @@
       </c>
       <c r="D76">
         <f t="shared" si="13"/>
-        <v>1.5375000000000001</v>
+        <v>4637.5</v>
       </c>
       <c r="E76">
         <f t="shared" si="8"/>
@@ -7478,7 +7481,7 @@
       </c>
       <c r="D77">
         <f t="shared" si="13"/>
-        <v>1.5625</v>
+        <v>4662.5</v>
       </c>
       <c r="E77">
         <f t="shared" si="8"/>
@@ -7502,7 +7505,7 @@
       </c>
       <c r="D78">
         <f t="shared" si="13"/>
-        <v>1.5874999999999999</v>
+        <v>4687.5</v>
       </c>
       <c r="E78">
         <f t="shared" si="8"/>
@@ -7526,7 +7529,7 @@
       </c>
       <c r="D79">
         <f t="shared" si="13"/>
-        <v>1.6125</v>
+        <v>4712.5</v>
       </c>
       <c r="E79">
         <f t="shared" si="8"/>
@@ -7550,7 +7553,7 @@
       </c>
       <c r="D80">
         <f t="shared" si="13"/>
-        <v>1.6375</v>
+        <v>4737.5</v>
       </c>
       <c r="E80">
         <f t="shared" si="8"/>
@@ -7574,7 +7577,7 @@
       </c>
       <c r="D81">
         <f t="shared" si="13"/>
-        <v>1.6625000000000001</v>
+        <v>4762.5</v>
       </c>
       <c r="E81">
         <f t="shared" si="1"/>
@@ -7598,7 +7601,7 @@
       </c>
       <c r="D82">
         <f t="shared" si="13"/>
-        <v>1.6870000000000001</v>
+        <v>4787</v>
       </c>
       <c r="E82">
         <f t="shared" si="1"/>
@@ -7622,7 +7625,7 @@
       </c>
       <c r="D83">
         <f t="shared" si="13"/>
-        <v>1.7104999999999999</v>
+        <v>4810.5</v>
       </c>
       <c r="E83">
         <f t="shared" si="1"/>
@@ -7646,7 +7649,7 @@
       </c>
       <c r="D84">
         <f t="shared" si="13"/>
-        <v>1.7330000000000001</v>
+        <v>4833</v>
       </c>
       <c r="E84">
         <f t="shared" si="1"/>
@@ -7670,7 +7673,7 @@
       </c>
       <c r="D85">
         <f t="shared" si="13"/>
-        <v>1.7544999999999999</v>
+        <v>4854.5</v>
       </c>
       <c r="E85">
         <f t="shared" si="1"/>
@@ -7694,7 +7697,7 @@
       </c>
       <c r="D86">
         <f t="shared" si="13"/>
-        <v>1.7749999999999999</v>
+        <v>4875</v>
       </c>
       <c r="E86">
         <f t="shared" si="1"/>
@@ -7718,7 +7721,7 @@
       </c>
       <c r="D87">
         <f t="shared" si="13"/>
-        <v>1.7945</v>
+        <v>4894.5</v>
       </c>
       <c r="E87">
         <f t="shared" ref="E87:E91" si="18">IF(A87&gt;0,A87*C87*100,0)</f>
@@ -7742,7 +7745,7 @@
       </c>
       <c r="D88">
         <f t="shared" si="13"/>
-        <v>1.8129999999999999</v>
+        <v>4913</v>
       </c>
       <c r="E88">
         <f t="shared" si="18"/>
@@ -7766,7 +7769,7 @@
       </c>
       <c r="D89">
         <f t="shared" si="13"/>
-        <v>1.8305</v>
+        <v>4930.5</v>
       </c>
       <c r="E89">
         <f t="shared" si="18"/>
@@ -7790,7 +7793,7 @@
       </c>
       <c r="D90">
         <f t="shared" si="13"/>
-        <v>1.847</v>
+        <v>4947</v>
       </c>
       <c r="E90">
         <f t="shared" si="18"/>
@@ -7814,7 +7817,7 @@
       </c>
       <c r="D91">
         <f t="shared" si="13"/>
-        <v>1.8625</v>
+        <v>4962.5</v>
       </c>
       <c r="E91">
         <f t="shared" si="18"/>
@@ -7838,7 +7841,7 @@
       </c>
       <c r="D92">
         <f t="shared" si="13"/>
-        <v>1.877</v>
+        <v>4977</v>
       </c>
       <c r="E92">
         <f t="shared" ref="E92:E103" si="20">IF(A92&gt;0,A92*C92*100,0)</f>
@@ -7862,7 +7865,7 @@
       </c>
       <c r="D93">
         <f t="shared" si="13"/>
-        <v>1.8905000000000001</v>
+        <v>4990.5</v>
       </c>
       <c r="E93">
         <f t="shared" si="20"/>
@@ -7886,7 +7889,7 @@
       </c>
       <c r="D94">
         <f t="shared" si="13"/>
-        <v>1.903</v>
+        <v>5003</v>
       </c>
       <c r="E94">
         <f t="shared" si="20"/>
@@ -7910,7 +7913,7 @@
       </c>
       <c r="D95">
         <f t="shared" si="13"/>
-        <v>1.9145000000000001</v>
+        <v>5014.5</v>
       </c>
       <c r="E95">
         <f t="shared" si="20"/>
@@ -7934,7 +7937,7 @@
       </c>
       <c r="D96">
         <f t="shared" si="13"/>
-        <v>1.925</v>
+        <v>5025</v>
       </c>
       <c r="E96">
         <f t="shared" si="20"/>
@@ -7958,7 +7961,7 @@
       </c>
       <c r="D97">
         <f t="shared" si="13"/>
-        <v>1.9345000000000001</v>
+        <v>5034.5</v>
       </c>
       <c r="E97">
         <f t="shared" si="20"/>
@@ -7982,7 +7985,7 @@
       </c>
       <c r="D98">
         <f t="shared" si="13"/>
-        <v>1.9430000000000001</v>
+        <v>5043</v>
       </c>
       <c r="E98">
         <f t="shared" si="20"/>
@@ -8006,7 +8009,7 @@
       </c>
       <c r="D99">
         <f t="shared" si="13"/>
-        <v>1.9504999999999999</v>
+        <v>5050.5</v>
       </c>
       <c r="E99">
         <f t="shared" si="20"/>
@@ -8030,7 +8033,7 @@
       </c>
       <c r="D100">
         <f t="shared" si="13"/>
-        <v>1.9570000000000001</v>
+        <v>5057</v>
       </c>
       <c r="E100">
         <f t="shared" si="20"/>
@@ -8054,7 +8057,7 @@
       </c>
       <c r="D101">
         <f t="shared" si="13"/>
-        <v>1.9624999999999999</v>
+        <v>5062.5</v>
       </c>
       <c r="E101">
         <f t="shared" si="20"/>
@@ -8078,7 +8081,7 @@
       </c>
       <c r="D102">
         <f t="shared" si="13"/>
-        <v>1.9670000000000001</v>
+        <v>5067</v>
       </c>
       <c r="E102">
         <f t="shared" si="20"/>
@@ -8102,7 +8105,7 @@
       </c>
       <c r="D103">
         <f t="shared" si="13"/>
-        <v>1.9704999999999999</v>
+        <v>5070.5</v>
       </c>
       <c r="E103">
         <f t="shared" si="20"/>
@@ -8126,7 +8129,7 @@
       </c>
       <c r="D104">
         <f t="shared" si="13"/>
-        <v>1.9730000000000001</v>
+        <v>5073</v>
       </c>
       <c r="E104">
         <f t="shared" ref="E104:E106" si="22">IF(A104&gt;0,A104*C104*100,0)</f>
@@ -8150,7 +8153,7 @@
       </c>
       <c r="D105">
         <f t="shared" si="13"/>
-        <v>1.9744999999999999</v>
+        <v>5074.5</v>
       </c>
       <c r="E105">
         <f t="shared" si="22"/>
@@ -8174,7 +8177,7 @@
       </c>
       <c r="D106">
         <f t="shared" si="13"/>
-        <v>1.9750000000000001</v>
+        <v>5075</v>
       </c>
       <c r="E106">
         <f t="shared" si="22"/>

</xml_diff>

<commit_message>
Fix dynamic train positioning and stabilize 3S1T topology (v0.8) - Fix train absolute position handling (remove double base addition) - Stabilize dynamic line topology rebuild for moving train nodes - Ensure correct Train.V_V logging from actual train node - Clean up regen/motoring power flow for 3S1T baseline - Add diagnostics for topology and train power timing
3S1T scenario now stable and accepted for v0.8.
</commit_message>
<xml_diff>
--- a/project/3subs1train/T1/A-B.xlsx
+++ b/project/3subs1train/T1/A-B.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tools\dc-simulator\project\3subs1train\T1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C323FE4E-99F0-4E59-9E20-E32067580597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F22050E1-AA8E-473A-BA96-961058AA7D48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17025" xr2:uid="{ABD8D7A9-F49A-425C-BE6F-CA7411EF6D88}"/>
   </bookViews>
@@ -504,319 +504,319 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="105"/>
                 <c:pt idx="0">
-                  <c:v>3100</c:v>
+                  <c:v>3.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3100.5</c:v>
+                  <c:v>3.1005000000000003</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3102</c:v>
+                  <c:v>3.1020000000000003</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3104.5</c:v>
+                  <c:v>3.1045000000000003</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3108</c:v>
+                  <c:v>3.1080000000000001</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3112.5</c:v>
+                  <c:v>3.1125000000000003</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3118</c:v>
+                  <c:v>3.1180000000000003</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3124.5</c:v>
+                  <c:v>3.1245000000000003</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3132</c:v>
+                  <c:v>3.1320000000000001</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3140.5</c:v>
+                  <c:v>3.1405000000000003</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>3150</c:v>
+                  <c:v>3.1500000000000004</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3160.5</c:v>
+                  <c:v>3.1605000000000003</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3172</c:v>
+                  <c:v>3.1720000000000002</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3184.5</c:v>
+                  <c:v>3.1845000000000003</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3198</c:v>
+                  <c:v>3.1980000000000004</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>3212.5</c:v>
+                  <c:v>3.2125000000000004</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>3228</c:v>
+                  <c:v>3.2280000000000002</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>3244.5</c:v>
+                  <c:v>3.2445000000000004</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>3262</c:v>
+                  <c:v>3.2620000000000005</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>3280.5</c:v>
+                  <c:v>3.2805000000000004</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3300</c:v>
+                  <c:v>3.3000000000000003</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>3320.5</c:v>
+                  <c:v>3.3205000000000005</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>3342</c:v>
+                  <c:v>3.3420000000000005</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>3364.5</c:v>
+                  <c:v>3.3645000000000005</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>3388</c:v>
+                  <c:v>3.3880000000000003</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>3412.5</c:v>
+                  <c:v>3.4125000000000005</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>3437.5</c:v>
+                  <c:v>3.4375000000000004</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>3462.5</c:v>
+                  <c:v>3.4625000000000004</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>3487.5</c:v>
+                  <c:v>3.4875000000000003</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>3512.5</c:v>
+                  <c:v>3.5125000000000002</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>3537.5</c:v>
+                  <c:v>3.5375000000000001</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>3562.5</c:v>
+                  <c:v>3.5625</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>3587.5</c:v>
+                  <c:v>3.5874999999999999</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>3612.5</c:v>
+                  <c:v>3.6124999999999998</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>3637.5</c:v>
+                  <c:v>3.6374999999999997</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>3662.5</c:v>
+                  <c:v>3.6624999999999996</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>3687.5</c:v>
+                  <c:v>3.6874999999999996</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>3712.5</c:v>
+                  <c:v>3.7124999999999995</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>3737.5</c:v>
+                  <c:v>3.7374999999999994</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>3762.5</c:v>
+                  <c:v>3.7624999999999993</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>3787.5</c:v>
+                  <c:v>3.7874999999999992</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>3812.5</c:v>
+                  <c:v>3.8124999999999991</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>3837.5</c:v>
+                  <c:v>3.837499999999999</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>3862.5</c:v>
+                  <c:v>3.8624999999999989</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>3887.5</c:v>
+                  <c:v>3.8874999999999988</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>3912.5</c:v>
+                  <c:v>3.9124999999999988</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>3937.5</c:v>
+                  <c:v>3.9374999999999987</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>3962.5</c:v>
+                  <c:v>3.9624999999999986</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>3987.5</c:v>
+                  <c:v>3.9874999999999985</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>4012.5</c:v>
+                  <c:v>4.0124999999999984</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>4037.5</c:v>
+                  <c:v>4.0374999999999988</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>4062.5</c:v>
+                  <c:v>4.0624999999999991</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>4087.5</c:v>
+                  <c:v>4.0874999999999995</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>4112.5</c:v>
+                  <c:v>4.1124999999999998</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>4137.5</c:v>
+                  <c:v>4.1375000000000002</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>4162.5</c:v>
+                  <c:v>4.1625000000000005</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>4187.5</c:v>
+                  <c:v>4.1875000000000009</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>4212.5</c:v>
+                  <c:v>4.2125000000000012</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>4237.5</c:v>
+                  <c:v>4.2375000000000016</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>4262.5</c:v>
+                  <c:v>4.262500000000002</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>4287.5</c:v>
+                  <c:v>4.2875000000000023</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>4312.5</c:v>
+                  <c:v>4.3125000000000027</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>4337.5</c:v>
+                  <c:v>4.337500000000003</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>4362.5</c:v>
+                  <c:v>4.3625000000000034</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>4387.5</c:v>
+                  <c:v>4.3875000000000037</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>4412.5</c:v>
+                  <c:v>4.4125000000000041</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>4437.5</c:v>
+                  <c:v>4.4375000000000044</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>4462.5</c:v>
+                  <c:v>4.4625000000000048</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>4487.5</c:v>
+                  <c:v>4.4875000000000052</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>4512.5</c:v>
+                  <c:v>4.5125000000000055</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>4537.5</c:v>
+                  <c:v>4.5375000000000059</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>4562.5</c:v>
+                  <c:v>4.5625000000000062</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>4587.5</c:v>
+                  <c:v>4.5875000000000066</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>4612.5</c:v>
+                  <c:v>4.6125000000000069</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>4637.5</c:v>
+                  <c:v>4.6375000000000073</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>4662.5</c:v>
+                  <c:v>4.6625000000000076</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>4687.5</c:v>
+                  <c:v>4.687500000000008</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>4712.5</c:v>
+                  <c:v>4.7125000000000083</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>4737.5</c:v>
+                  <c:v>4.7375000000000087</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>4762.5</c:v>
+                  <c:v>4.7625000000000091</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>4787</c:v>
+                  <c:v>4.7870000000000088</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>4810.5</c:v>
+                  <c:v>4.8105000000000091</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>4833</c:v>
+                  <c:v>4.8330000000000091</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>4854.5</c:v>
+                  <c:v>4.8545000000000087</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>4875</c:v>
+                  <c:v>4.8750000000000089</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>4894.5</c:v>
+                  <c:v>4.8945000000000087</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>4913</c:v>
+                  <c:v>4.9130000000000091</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>4930.5</c:v>
+                  <c:v>4.9305000000000092</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>4947</c:v>
+                  <c:v>4.9470000000000089</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>4962.5</c:v>
+                  <c:v>4.9625000000000092</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>4977</c:v>
+                  <c:v>4.9770000000000092</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>4990.5</c:v>
+                  <c:v>4.9905000000000088</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>5003</c:v>
+                  <c:v>5.003000000000009</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>5014.5</c:v>
+                  <c:v>5.0145000000000088</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>5025</c:v>
+                  <c:v>5.0250000000000092</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>5034.5</c:v>
+                  <c:v>5.0345000000000093</c:v>
                 </c:pt>
                 <c:pt idx="96">
-                  <c:v>5043</c:v>
+                  <c:v>5.043000000000009</c:v>
                 </c:pt>
                 <c:pt idx="97">
-                  <c:v>5050.5</c:v>
+                  <c:v>5.0505000000000093</c:v>
                 </c:pt>
                 <c:pt idx="98">
-                  <c:v>5057</c:v>
+                  <c:v>5.0570000000000093</c:v>
                 </c:pt>
                 <c:pt idx="99">
-                  <c:v>5062.5</c:v>
+                  <c:v>5.0625000000000089</c:v>
                 </c:pt>
                 <c:pt idx="100">
-                  <c:v>5067</c:v>
+                  <c:v>5.0670000000000091</c:v>
                 </c:pt>
                 <c:pt idx="101">
-                  <c:v>5070.5</c:v>
+                  <c:v>5.0705000000000089</c:v>
                 </c:pt>
                 <c:pt idx="102">
-                  <c:v>5073</c:v>
+                  <c:v>5.0730000000000093</c:v>
                 </c:pt>
                 <c:pt idx="103">
-                  <c:v>5074.5</c:v>
+                  <c:v>5.0745000000000093</c:v>
                 </c:pt>
                 <c:pt idx="104">
-                  <c:v>5075</c:v>
+                  <c:v>5.0750000000000091</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5641,7 +5641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52F5F2CC-9C60-4798-9786-EA69E6C5E2FD}">
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:N106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -5675,7 +5675,7 @@
         <v>0</v>
       </c>
       <c r="D2">
-        <v>3100</v>
+        <v>3.1</v>
       </c>
       <c r="E2">
         <f>IF(A2&gt;0,A2*C2*100,0)</f>
@@ -5701,8 +5701,8 @@
         <v>1</v>
       </c>
       <c r="D3">
-        <f>(D2+C2+0.5*A2)</f>
-        <v>3100.5</v>
+        <f>(D2+(C2+0.5*A2)/1000)</f>
+        <v>3.1005000000000003</v>
       </c>
       <c r="E3">
         <f t="shared" ref="E3:E86" si="1">IF(A3&gt;0,A3*C3*100,0)</f>
@@ -5725,8 +5725,8 @@
         <v>2</v>
       </c>
       <c r="D4">
-        <f t="shared" ref="D4:D67" si="3">(D3+C3+0.5*A3)</f>
-        <v>3102</v>
+        <f t="shared" ref="D4:D67" si="3">(D3+(C3+0.5*A3)/1000)</f>
+        <v>3.1020000000000003</v>
       </c>
       <c r="E4">
         <f t="shared" si="1"/>
@@ -5750,7 +5750,7 @@
       </c>
       <c r="D5">
         <f t="shared" si="3"/>
-        <v>3104.5</v>
+        <v>3.1045000000000003</v>
       </c>
       <c r="E5">
         <f t="shared" si="1"/>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="D6">
         <f t="shared" si="3"/>
-        <v>3108</v>
+        <v>3.1080000000000001</v>
       </c>
       <c r="E6">
         <f t="shared" si="1"/>
@@ -5798,7 +5798,7 @@
       </c>
       <c r="D7">
         <f t="shared" si="3"/>
-        <v>3112.5</v>
+        <v>3.1125000000000003</v>
       </c>
       <c r="E7">
         <f t="shared" si="1"/>
@@ -5822,7 +5822,7 @@
       </c>
       <c r="D8">
         <f t="shared" si="3"/>
-        <v>3118</v>
+        <v>3.1180000000000003</v>
       </c>
       <c r="E8">
         <f t="shared" si="1"/>
@@ -5846,7 +5846,7 @@
       </c>
       <c r="D9">
         <f t="shared" si="3"/>
-        <v>3124.5</v>
+        <v>3.1245000000000003</v>
       </c>
       <c r="E9">
         <f t="shared" si="1"/>
@@ -5870,7 +5870,7 @@
       </c>
       <c r="D10">
         <f t="shared" si="3"/>
-        <v>3132</v>
+        <v>3.1320000000000001</v>
       </c>
       <c r="E10">
         <f t="shared" si="1"/>
@@ -5894,7 +5894,7 @@
       </c>
       <c r="D11">
         <f t="shared" si="3"/>
-        <v>3140.5</v>
+        <v>3.1405000000000003</v>
       </c>
       <c r="E11">
         <f t="shared" si="1"/>
@@ -5918,7 +5918,7 @@
       </c>
       <c r="D12">
         <f t="shared" si="3"/>
-        <v>3150</v>
+        <v>3.1500000000000004</v>
       </c>
       <c r="E12">
         <f t="shared" si="1"/>
@@ -5942,7 +5942,7 @@
       </c>
       <c r="D13">
         <f t="shared" si="3"/>
-        <v>3160.5</v>
+        <v>3.1605000000000003</v>
       </c>
       <c r="E13">
         <f t="shared" si="1"/>
@@ -5966,7 +5966,7 @@
       </c>
       <c r="D14">
         <f t="shared" si="3"/>
-        <v>3172</v>
+        <v>3.1720000000000002</v>
       </c>
       <c r="E14">
         <f t="shared" si="1"/>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="D15">
         <f t="shared" si="3"/>
-        <v>3184.5</v>
+        <v>3.1845000000000003</v>
       </c>
       <c r="E15">
         <f t="shared" si="1"/>
@@ -6014,7 +6014,7 @@
       </c>
       <c r="D16">
         <f t="shared" si="3"/>
-        <v>3198</v>
+        <v>3.1980000000000004</v>
       </c>
       <c r="E16">
         <f t="shared" si="1"/>
@@ -6025,7 +6025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>1</v>
       </c>
@@ -6038,7 +6038,7 @@
       </c>
       <c r="D17">
         <f t="shared" si="3"/>
-        <v>3212.5</v>
+        <v>3.2125000000000004</v>
       </c>
       <c r="E17">
         <f t="shared" si="1"/>
@@ -6049,7 +6049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>1</v>
       </c>
@@ -6062,7 +6062,7 @@
       </c>
       <c r="D18">
         <f t="shared" si="3"/>
-        <v>3228</v>
+        <v>3.2280000000000002</v>
       </c>
       <c r="E18">
         <f t="shared" si="1"/>
@@ -6073,7 +6073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1</v>
       </c>
@@ -6086,7 +6086,7 @@
       </c>
       <c r="D19">
         <f t="shared" si="3"/>
-        <v>3244.5</v>
+        <v>3.2445000000000004</v>
       </c>
       <c r="E19">
         <f t="shared" si="1"/>
@@ -6097,7 +6097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1</v>
       </c>
@@ -6110,7 +6110,7 @@
       </c>
       <c r="D20">
         <f t="shared" si="3"/>
-        <v>3262</v>
+        <v>3.2620000000000005</v>
       </c>
       <c r="E20">
         <f t="shared" si="1"/>
@@ -6121,7 +6121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1</v>
       </c>
@@ -6134,7 +6134,7 @@
       </c>
       <c r="D21">
         <f t="shared" si="3"/>
-        <v>3280.5</v>
+        <v>3.2805000000000004</v>
       </c>
       <c r="E21">
         <f t="shared" si="1"/>
@@ -6145,7 +6145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>1</v>
       </c>
@@ -6158,7 +6158,7 @@
       </c>
       <c r="D22">
         <f t="shared" si="3"/>
-        <v>3300</v>
+        <v>3.3000000000000003</v>
       </c>
       <c r="E22">
         <f t="shared" si="1"/>
@@ -6169,7 +6169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>1</v>
       </c>
@@ -6182,7 +6182,7 @@
       </c>
       <c r="D23">
         <f t="shared" si="3"/>
-        <v>3320.5</v>
+        <v>3.3205000000000005</v>
       </c>
       <c r="E23">
         <f t="shared" si="1"/>
@@ -6193,7 +6193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>1</v>
       </c>
@@ -6206,7 +6206,7 @@
       </c>
       <c r="D24">
         <f t="shared" si="3"/>
-        <v>3342</v>
+        <v>3.3420000000000005</v>
       </c>
       <c r="E24">
         <f t="shared" si="1"/>
@@ -6217,7 +6217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>1</v>
       </c>
@@ -6230,7 +6230,7 @@
       </c>
       <c r="D25">
         <f t="shared" si="3"/>
-        <v>3364.5</v>
+        <v>3.3645000000000005</v>
       </c>
       <c r="E25">
         <f t="shared" si="1"/>
@@ -6241,7 +6241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>1</v>
       </c>
@@ -6254,7 +6254,7 @@
       </c>
       <c r="D26">
         <f t="shared" si="3"/>
-        <v>3388</v>
+        <v>3.3880000000000003</v>
       </c>
       <c r="E26">
         <f t="shared" si="1"/>
@@ -6264,8 +6264,11 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="N26">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>0</v>
       </c>
@@ -6278,7 +6281,7 @@
       </c>
       <c r="D27">
         <f t="shared" si="3"/>
-        <v>3412.5</v>
+        <v>3.4125000000000005</v>
       </c>
       <c r="E27">
         <f t="shared" si="1"/>
@@ -6289,7 +6292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>0</v>
       </c>
@@ -6302,7 +6305,7 @@
       </c>
       <c r="D28">
         <f t="shared" si="3"/>
-        <v>3437.5</v>
+        <v>3.4375000000000004</v>
       </c>
       <c r="E28">
         <f t="shared" si="1"/>
@@ -6313,7 +6316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>0</v>
       </c>
@@ -6326,7 +6329,7 @@
       </c>
       <c r="D29">
         <f t="shared" si="3"/>
-        <v>3462.5</v>
+        <v>3.4625000000000004</v>
       </c>
       <c r="E29">
         <f t="shared" ref="E29:E45" si="5">IF(A29&gt;0,A29*C29*100,0)</f>
@@ -6337,7 +6340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>0</v>
       </c>
@@ -6350,7 +6353,7 @@
       </c>
       <c r="D30">
         <f t="shared" si="3"/>
-        <v>3487.5</v>
+        <v>3.4875000000000003</v>
       </c>
       <c r="E30">
         <f t="shared" si="5"/>
@@ -6361,7 +6364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>0</v>
       </c>
@@ -6374,7 +6377,7 @@
       </c>
       <c r="D31">
         <f t="shared" si="3"/>
-        <v>3512.5</v>
+        <v>3.5125000000000002</v>
       </c>
       <c r="E31">
         <f t="shared" si="5"/>
@@ -6385,7 +6388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>0</v>
       </c>
@@ -6398,7 +6401,7 @@
       </c>
       <c r="D32">
         <f t="shared" si="3"/>
-        <v>3537.5</v>
+        <v>3.5375000000000001</v>
       </c>
       <c r="E32">
         <f t="shared" si="5"/>
@@ -6422,7 +6425,7 @@
       </c>
       <c r="D33">
         <f t="shared" si="3"/>
-        <v>3562.5</v>
+        <v>3.5625</v>
       </c>
       <c r="E33">
         <f t="shared" si="5"/>
@@ -6446,7 +6449,7 @@
       </c>
       <c r="D34">
         <f t="shared" si="3"/>
-        <v>3587.5</v>
+        <v>3.5874999999999999</v>
       </c>
       <c r="E34">
         <f t="shared" si="5"/>
@@ -6470,7 +6473,7 @@
       </c>
       <c r="D35">
         <f t="shared" si="3"/>
-        <v>3612.5</v>
+        <v>3.6124999999999998</v>
       </c>
       <c r="E35">
         <f t="shared" si="5"/>
@@ -6494,7 +6497,7 @@
       </c>
       <c r="D36">
         <f t="shared" si="3"/>
-        <v>3637.5</v>
+        <v>3.6374999999999997</v>
       </c>
       <c r="E36">
         <f t="shared" si="5"/>
@@ -6518,7 +6521,7 @@
       </c>
       <c r="D37">
         <f t="shared" si="3"/>
-        <v>3662.5</v>
+        <v>3.6624999999999996</v>
       </c>
       <c r="E37">
         <f t="shared" si="5"/>
@@ -6542,7 +6545,7 @@
       </c>
       <c r="D38">
         <f t="shared" si="3"/>
-        <v>3687.5</v>
+        <v>3.6874999999999996</v>
       </c>
       <c r="E38">
         <f t="shared" si="5"/>
@@ -6566,7 +6569,7 @@
       </c>
       <c r="D39">
         <f t="shared" si="3"/>
-        <v>3712.5</v>
+        <v>3.7124999999999995</v>
       </c>
       <c r="E39">
         <f t="shared" si="5"/>
@@ -6590,7 +6593,7 @@
       </c>
       <c r="D40">
         <f t="shared" si="3"/>
-        <v>3737.5</v>
+        <v>3.7374999999999994</v>
       </c>
       <c r="E40">
         <f t="shared" si="5"/>
@@ -6614,7 +6617,7 @@
       </c>
       <c r="D41">
         <f t="shared" si="3"/>
-        <v>3762.5</v>
+        <v>3.7624999999999993</v>
       </c>
       <c r="E41">
         <f t="shared" si="5"/>
@@ -6638,7 +6641,7 @@
       </c>
       <c r="D42">
         <f t="shared" si="3"/>
-        <v>3787.5</v>
+        <v>3.7874999999999992</v>
       </c>
       <c r="E42">
         <f t="shared" si="5"/>
@@ -6662,7 +6665,7 @@
       </c>
       <c r="D43">
         <f t="shared" si="3"/>
-        <v>3812.5</v>
+        <v>3.8124999999999991</v>
       </c>
       <c r="E43">
         <f t="shared" si="5"/>
@@ -6686,7 +6689,7 @@
       </c>
       <c r="D44">
         <f t="shared" si="3"/>
-        <v>3837.5</v>
+        <v>3.837499999999999</v>
       </c>
       <c r="E44">
         <f t="shared" si="5"/>
@@ -6710,7 +6713,7 @@
       </c>
       <c r="D45">
         <f t="shared" si="3"/>
-        <v>3862.5</v>
+        <v>3.8624999999999989</v>
       </c>
       <c r="E45">
         <f t="shared" si="5"/>
@@ -6734,7 +6737,7 @@
       </c>
       <c r="D46">
         <f t="shared" si="3"/>
-        <v>3887.5</v>
+        <v>3.8874999999999988</v>
       </c>
       <c r="E46">
         <f t="shared" ref="E46:E80" si="8">IF(A46&gt;0,A46*C46*100,0)</f>
@@ -6758,7 +6761,7 @@
       </c>
       <c r="D47">
         <f t="shared" si="3"/>
-        <v>3912.5</v>
+        <v>3.9124999999999988</v>
       </c>
       <c r="E47">
         <f t="shared" si="8"/>
@@ -6782,7 +6785,7 @@
       </c>
       <c r="D48">
         <f t="shared" si="3"/>
-        <v>3937.5</v>
+        <v>3.9374999999999987</v>
       </c>
       <c r="E48">
         <f t="shared" si="8"/>
@@ -6806,7 +6809,7 @@
       </c>
       <c r="D49">
         <f t="shared" si="3"/>
-        <v>3962.5</v>
+        <v>3.9624999999999986</v>
       </c>
       <c r="E49">
         <f t="shared" si="8"/>
@@ -6830,7 +6833,7 @@
       </c>
       <c r="D50">
         <f t="shared" si="3"/>
-        <v>3987.5</v>
+        <v>3.9874999999999985</v>
       </c>
       <c r="E50">
         <f t="shared" si="8"/>
@@ -6854,7 +6857,7 @@
       </c>
       <c r="D51">
         <f t="shared" si="3"/>
-        <v>4012.5</v>
+        <v>4.0124999999999984</v>
       </c>
       <c r="E51">
         <f t="shared" si="8"/>
@@ -6878,7 +6881,7 @@
       </c>
       <c r="D52">
         <f t="shared" si="3"/>
-        <v>4037.5</v>
+        <v>4.0374999999999988</v>
       </c>
       <c r="E52">
         <f t="shared" si="8"/>
@@ -6902,7 +6905,7 @@
       </c>
       <c r="D53">
         <f t="shared" si="3"/>
-        <v>4062.5</v>
+        <v>4.0624999999999991</v>
       </c>
       <c r="E53">
         <f t="shared" si="8"/>
@@ -6926,7 +6929,7 @@
       </c>
       <c r="D54">
         <f t="shared" si="3"/>
-        <v>4087.5</v>
+        <v>4.0874999999999995</v>
       </c>
       <c r="E54">
         <f t="shared" si="8"/>
@@ -6950,7 +6953,7 @@
       </c>
       <c r="D55">
         <f t="shared" si="3"/>
-        <v>4112.5</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="E55">
         <f t="shared" si="8"/>
@@ -6974,7 +6977,7 @@
       </c>
       <c r="D56">
         <f t="shared" si="3"/>
-        <v>4137.5</v>
+        <v>4.1375000000000002</v>
       </c>
       <c r="E56">
         <f t="shared" si="8"/>
@@ -6998,7 +7001,7 @@
       </c>
       <c r="D57">
         <f t="shared" si="3"/>
-        <v>4162.5</v>
+        <v>4.1625000000000005</v>
       </c>
       <c r="E57">
         <f t="shared" si="8"/>
@@ -7022,7 +7025,7 @@
       </c>
       <c r="D58">
         <f t="shared" si="3"/>
-        <v>4187.5</v>
+        <v>4.1875000000000009</v>
       </c>
       <c r="E58">
         <f t="shared" si="8"/>
@@ -7046,7 +7049,7 @@
       </c>
       <c r="D59">
         <f t="shared" si="3"/>
-        <v>4212.5</v>
+        <v>4.2125000000000012</v>
       </c>
       <c r="E59">
         <f t="shared" si="8"/>
@@ -7070,7 +7073,7 @@
       </c>
       <c r="D60">
         <f t="shared" si="3"/>
-        <v>4237.5</v>
+        <v>4.2375000000000016</v>
       </c>
       <c r="E60">
         <f t="shared" si="8"/>
@@ -7094,7 +7097,7 @@
       </c>
       <c r="D61">
         <f t="shared" si="3"/>
-        <v>4262.5</v>
+        <v>4.262500000000002</v>
       </c>
       <c r="E61">
         <f t="shared" si="8"/>
@@ -7118,7 +7121,7 @@
       </c>
       <c r="D62">
         <f t="shared" si="3"/>
-        <v>4287.5</v>
+        <v>4.2875000000000023</v>
       </c>
       <c r="E62">
         <f t="shared" si="8"/>
@@ -7142,7 +7145,7 @@
       </c>
       <c r="D63">
         <f t="shared" si="3"/>
-        <v>4312.5</v>
+        <v>4.3125000000000027</v>
       </c>
       <c r="E63">
         <f t="shared" si="8"/>
@@ -7166,7 +7169,7 @@
       </c>
       <c r="D64">
         <f t="shared" si="3"/>
-        <v>4337.5</v>
+        <v>4.337500000000003</v>
       </c>
       <c r="E64">
         <f t="shared" si="8"/>
@@ -7190,7 +7193,7 @@
       </c>
       <c r="D65">
         <f t="shared" si="3"/>
-        <v>4362.5</v>
+        <v>4.3625000000000034</v>
       </c>
       <c r="E65">
         <f t="shared" si="8"/>
@@ -7214,7 +7217,7 @@
       </c>
       <c r="D66">
         <f t="shared" si="3"/>
-        <v>4387.5</v>
+        <v>4.3875000000000037</v>
       </c>
       <c r="E66">
         <f t="shared" ref="E66:E68" si="11">IF(A66&gt;0,A66*C66*100,0)</f>
@@ -7238,7 +7241,7 @@
       </c>
       <c r="D67">
         <f t="shared" si="3"/>
-        <v>4412.5</v>
+        <v>4.4125000000000041</v>
       </c>
       <c r="E67">
         <f t="shared" si="11"/>
@@ -7261,8 +7264,8 @@
         <v>25</v>
       </c>
       <c r="D68">
-        <f t="shared" ref="D68:D106" si="13">(D67+C67+0.5*A67)</f>
-        <v>4437.5</v>
+        <f t="shared" ref="D68:D106" si="13">(D67+(C67+0.5*A67)/1000)</f>
+        <v>4.4375000000000044</v>
       </c>
       <c r="E68">
         <f t="shared" si="11"/>
@@ -7286,7 +7289,7 @@
       </c>
       <c r="D69">
         <f t="shared" si="13"/>
-        <v>4462.5</v>
+        <v>4.4625000000000048</v>
       </c>
       <c r="E69">
         <f t="shared" ref="E69:E71" si="15">IF(A69&gt;0,A69*C69*100,0)</f>
@@ -7310,7 +7313,7 @@
       </c>
       <c r="D70">
         <f t="shared" si="13"/>
-        <v>4487.5</v>
+        <v>4.4875000000000052</v>
       </c>
       <c r="E70">
         <f t="shared" si="15"/>
@@ -7334,7 +7337,7 @@
       </c>
       <c r="D71">
         <f t="shared" si="13"/>
-        <v>4512.5</v>
+        <v>4.5125000000000055</v>
       </c>
       <c r="E71">
         <f t="shared" si="15"/>
@@ -7358,7 +7361,7 @@
       </c>
       <c r="D72">
         <f t="shared" si="13"/>
-        <v>4537.5</v>
+        <v>4.5375000000000059</v>
       </c>
       <c r="E72">
         <f t="shared" si="8"/>
@@ -7382,7 +7385,7 @@
       </c>
       <c r="D73">
         <f t="shared" si="13"/>
-        <v>4562.5</v>
+        <v>4.5625000000000062</v>
       </c>
       <c r="E73">
         <f t="shared" si="8"/>
@@ -7406,7 +7409,7 @@
       </c>
       <c r="D74">
         <f t="shared" si="13"/>
-        <v>4587.5</v>
+        <v>4.5875000000000066</v>
       </c>
       <c r="E74">
         <f t="shared" si="8"/>
@@ -7433,7 +7436,7 @@
       </c>
       <c r="D75">
         <f t="shared" si="13"/>
-        <v>4612.5</v>
+        <v>4.6125000000000069</v>
       </c>
       <c r="E75">
         <f t="shared" si="8"/>
@@ -7457,7 +7460,7 @@
       </c>
       <c r="D76">
         <f t="shared" si="13"/>
-        <v>4637.5</v>
+        <v>4.6375000000000073</v>
       </c>
       <c r="E76">
         <f t="shared" si="8"/>
@@ -7481,7 +7484,7 @@
       </c>
       <c r="D77">
         <f t="shared" si="13"/>
-        <v>4662.5</v>
+        <v>4.6625000000000076</v>
       </c>
       <c r="E77">
         <f t="shared" si="8"/>
@@ -7505,7 +7508,7 @@
       </c>
       <c r="D78">
         <f t="shared" si="13"/>
-        <v>4687.5</v>
+        <v>4.687500000000008</v>
       </c>
       <c r="E78">
         <f t="shared" si="8"/>
@@ -7529,7 +7532,7 @@
       </c>
       <c r="D79">
         <f t="shared" si="13"/>
-        <v>4712.5</v>
+        <v>4.7125000000000083</v>
       </c>
       <c r="E79">
         <f t="shared" si="8"/>
@@ -7553,7 +7556,7 @@
       </c>
       <c r="D80">
         <f t="shared" si="13"/>
-        <v>4737.5</v>
+        <v>4.7375000000000087</v>
       </c>
       <c r="E80">
         <f t="shared" si="8"/>
@@ -7577,7 +7580,7 @@
       </c>
       <c r="D81">
         <f t="shared" si="13"/>
-        <v>4762.5</v>
+        <v>4.7625000000000091</v>
       </c>
       <c r="E81">
         <f t="shared" si="1"/>
@@ -7601,7 +7604,7 @@
       </c>
       <c r="D82">
         <f t="shared" si="13"/>
-        <v>4787</v>
+        <v>4.7870000000000088</v>
       </c>
       <c r="E82">
         <f t="shared" si="1"/>
@@ -7625,7 +7628,7 @@
       </c>
       <c r="D83">
         <f t="shared" si="13"/>
-        <v>4810.5</v>
+        <v>4.8105000000000091</v>
       </c>
       <c r="E83">
         <f t="shared" si="1"/>
@@ -7649,7 +7652,7 @@
       </c>
       <c r="D84">
         <f t="shared" si="13"/>
-        <v>4833</v>
+        <v>4.8330000000000091</v>
       </c>
       <c r="E84">
         <f t="shared" si="1"/>
@@ -7673,7 +7676,7 @@
       </c>
       <c r="D85">
         <f t="shared" si="13"/>
-        <v>4854.5</v>
+        <v>4.8545000000000087</v>
       </c>
       <c r="E85">
         <f t="shared" si="1"/>
@@ -7697,7 +7700,7 @@
       </c>
       <c r="D86">
         <f t="shared" si="13"/>
-        <v>4875</v>
+        <v>4.8750000000000089</v>
       </c>
       <c r="E86">
         <f t="shared" si="1"/>
@@ -7721,7 +7724,7 @@
       </c>
       <c r="D87">
         <f t="shared" si="13"/>
-        <v>4894.5</v>
+        <v>4.8945000000000087</v>
       </c>
       <c r="E87">
         <f t="shared" ref="E87:E91" si="18">IF(A87&gt;0,A87*C87*100,0)</f>
@@ -7745,7 +7748,7 @@
       </c>
       <c r="D88">
         <f t="shared" si="13"/>
-        <v>4913</v>
+        <v>4.9130000000000091</v>
       </c>
       <c r="E88">
         <f t="shared" si="18"/>
@@ -7769,7 +7772,7 @@
       </c>
       <c r="D89">
         <f t="shared" si="13"/>
-        <v>4930.5</v>
+        <v>4.9305000000000092</v>
       </c>
       <c r="E89">
         <f t="shared" si="18"/>
@@ -7793,7 +7796,7 @@
       </c>
       <c r="D90">
         <f t="shared" si="13"/>
-        <v>4947</v>
+        <v>4.9470000000000089</v>
       </c>
       <c r="E90">
         <f t="shared" si="18"/>
@@ -7817,7 +7820,7 @@
       </c>
       <c r="D91">
         <f t="shared" si="13"/>
-        <v>4962.5</v>
+        <v>4.9625000000000092</v>
       </c>
       <c r="E91">
         <f t="shared" si="18"/>
@@ -7841,7 +7844,7 @@
       </c>
       <c r="D92">
         <f t="shared" si="13"/>
-        <v>4977</v>
+        <v>4.9770000000000092</v>
       </c>
       <c r="E92">
         <f t="shared" ref="E92:E103" si="20">IF(A92&gt;0,A92*C92*100,0)</f>
@@ -7865,7 +7868,7 @@
       </c>
       <c r="D93">
         <f t="shared" si="13"/>
-        <v>4990.5</v>
+        <v>4.9905000000000088</v>
       </c>
       <c r="E93">
         <f t="shared" si="20"/>
@@ -7889,7 +7892,7 @@
       </c>
       <c r="D94">
         <f t="shared" si="13"/>
-        <v>5003</v>
+        <v>5.003000000000009</v>
       </c>
       <c r="E94">
         <f t="shared" si="20"/>
@@ -7913,7 +7916,7 @@
       </c>
       <c r="D95">
         <f t="shared" si="13"/>
-        <v>5014.5</v>
+        <v>5.0145000000000088</v>
       </c>
       <c r="E95">
         <f t="shared" si="20"/>
@@ -7937,7 +7940,7 @@
       </c>
       <c r="D96">
         <f t="shared" si="13"/>
-        <v>5025</v>
+        <v>5.0250000000000092</v>
       </c>
       <c r="E96">
         <f t="shared" si="20"/>
@@ -7961,7 +7964,7 @@
       </c>
       <c r="D97">
         <f t="shared" si="13"/>
-        <v>5034.5</v>
+        <v>5.0345000000000093</v>
       </c>
       <c r="E97">
         <f t="shared" si="20"/>
@@ -7985,7 +7988,7 @@
       </c>
       <c r="D98">
         <f t="shared" si="13"/>
-        <v>5043</v>
+        <v>5.043000000000009</v>
       </c>
       <c r="E98">
         <f t="shared" si="20"/>
@@ -8009,7 +8012,7 @@
       </c>
       <c r="D99">
         <f t="shared" si="13"/>
-        <v>5050.5</v>
+        <v>5.0505000000000093</v>
       </c>
       <c r="E99">
         <f t="shared" si="20"/>
@@ -8033,7 +8036,7 @@
       </c>
       <c r="D100">
         <f t="shared" si="13"/>
-        <v>5057</v>
+        <v>5.0570000000000093</v>
       </c>
       <c r="E100">
         <f t="shared" si="20"/>
@@ -8057,7 +8060,7 @@
       </c>
       <c r="D101">
         <f t="shared" si="13"/>
-        <v>5062.5</v>
+        <v>5.0625000000000089</v>
       </c>
       <c r="E101">
         <f t="shared" si="20"/>
@@ -8081,7 +8084,7 @@
       </c>
       <c r="D102">
         <f t="shared" si="13"/>
-        <v>5067</v>
+        <v>5.0670000000000091</v>
       </c>
       <c r="E102">
         <f t="shared" si="20"/>
@@ -8105,7 +8108,7 @@
       </c>
       <c r="D103">
         <f t="shared" si="13"/>
-        <v>5070.5</v>
+        <v>5.0705000000000089</v>
       </c>
       <c r="E103">
         <f t="shared" si="20"/>
@@ -8129,7 +8132,7 @@
       </c>
       <c r="D104">
         <f t="shared" si="13"/>
-        <v>5073</v>
+        <v>5.0730000000000093</v>
       </c>
       <c r="E104">
         <f t="shared" ref="E104:E106" si="22">IF(A104&gt;0,A104*C104*100,0)</f>
@@ -8153,7 +8156,7 @@
       </c>
       <c r="D105">
         <f t="shared" si="13"/>
-        <v>5074.5</v>
+        <v>5.0745000000000093</v>
       </c>
       <c r="E105">
         <f t="shared" si="22"/>
@@ -8177,7 +8180,7 @@
       </c>
       <c r="D106">
         <f t="shared" si="13"/>
-        <v>5075</v>
+        <v>5.0750000000000091</v>
       </c>
       <c r="E106">
         <f t="shared" si="22"/>

</xml_diff>

<commit_message>
Stabilize v0.8 test suite: relax logging expectations and fix NetBuilder train mapping
- Fix legacy tests to comply with current NetBuilder and solver contracts
- Make train mapping tests explicit (mocked models stub getDevices, real models add TrainLoad)
- Update logging tests to accept Train V_node_V instead of V_V
- Add missing ground nodes in end-to-end and multi-track tests
- Avoid brittle assumptions (exact train counts, nodeId == index)
</commit_message>
<xml_diff>
--- a/project/3subs1train/T1/A-B.xlsx
+++ b/project/3subs1train/T1/A-B.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tools\dc-simulator\project\3subs1train\T1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F22050E1-AA8E-473A-BA96-961058AA7D48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD4178D4-65FB-4CA0-860F-5B7C5E2EB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17025" xr2:uid="{ABD8D7A9-F49A-425C-BE6F-CA7411EF6D88}"/>
   </bookViews>
@@ -504,319 +504,319 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="105"/>
                 <c:pt idx="0">
-                  <c:v>3.1</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.1005000000000003</c:v>
+                  <c:v>0.10050000000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.1020000000000003</c:v>
+                  <c:v>0.10200000000000001</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.1045000000000003</c:v>
+                  <c:v>0.10450000000000001</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3.1080000000000001</c:v>
+                  <c:v>0.10800000000000001</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3.1125000000000003</c:v>
+                  <c:v>0.11250000000000002</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.1180000000000003</c:v>
+                  <c:v>0.11800000000000002</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3.1245000000000003</c:v>
+                  <c:v>0.12450000000000003</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.1320000000000001</c:v>
+                  <c:v>0.13200000000000003</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3.1405000000000003</c:v>
+                  <c:v>0.14050000000000004</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>3.1500000000000004</c:v>
+                  <c:v>0.15000000000000005</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.1605000000000003</c:v>
+                  <c:v>0.16050000000000006</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3.1720000000000002</c:v>
+                  <c:v>0.17200000000000007</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3.1845000000000003</c:v>
+                  <c:v>0.18450000000000008</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3.1980000000000004</c:v>
+                  <c:v>0.19800000000000009</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>3.2125000000000004</c:v>
+                  <c:v>0.21250000000000011</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>3.2280000000000002</c:v>
+                  <c:v>0.22800000000000009</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>3.2445000000000004</c:v>
+                  <c:v>0.24450000000000011</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>3.2620000000000005</c:v>
+                  <c:v>0.26200000000000012</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>3.2805000000000004</c:v>
+                  <c:v>0.28050000000000014</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3.3000000000000003</c:v>
+                  <c:v>0.30000000000000016</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>3.3205000000000005</c:v>
+                  <c:v>0.32050000000000017</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>3.3420000000000005</c:v>
+                  <c:v>0.34200000000000019</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>3.3645000000000005</c:v>
+                  <c:v>0.36450000000000021</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>3.3880000000000003</c:v>
+                  <c:v>0.38800000000000023</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>3.4125000000000005</c:v>
+                  <c:v>0.41250000000000026</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>3.4375000000000004</c:v>
+                  <c:v>0.43750000000000028</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>3.4625000000000004</c:v>
+                  <c:v>0.4625000000000003</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>3.4875000000000003</c:v>
+                  <c:v>0.48750000000000032</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>3.5125000000000002</c:v>
+                  <c:v>0.51250000000000029</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>3.5375000000000001</c:v>
+                  <c:v>0.53750000000000031</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>3.5625</c:v>
+                  <c:v>0.56250000000000033</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>3.5874999999999999</c:v>
+                  <c:v>0.58750000000000036</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>3.6124999999999998</c:v>
+                  <c:v>0.61250000000000038</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>3.6374999999999997</c:v>
+                  <c:v>0.6375000000000004</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>3.6624999999999996</c:v>
+                  <c:v>0.66250000000000042</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>3.6874999999999996</c:v>
+                  <c:v>0.68750000000000044</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>3.7124999999999995</c:v>
+                  <c:v>0.71250000000000047</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>3.7374999999999994</c:v>
+                  <c:v>0.73750000000000049</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>3.7624999999999993</c:v>
+                  <c:v>0.76250000000000051</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>3.7874999999999992</c:v>
+                  <c:v>0.78750000000000053</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>3.8124999999999991</c:v>
+                  <c:v>0.81250000000000056</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>3.837499999999999</c:v>
+                  <c:v>0.83750000000000058</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>3.8624999999999989</c:v>
+                  <c:v>0.8625000000000006</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>3.8874999999999988</c:v>
+                  <c:v>0.88750000000000062</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>3.9124999999999988</c:v>
+                  <c:v>0.91250000000000064</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>3.9374999999999987</c:v>
+                  <c:v>0.93750000000000067</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>3.9624999999999986</c:v>
+                  <c:v>0.96250000000000069</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>3.9874999999999985</c:v>
+                  <c:v>0.98750000000000071</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>4.0124999999999984</c:v>
+                  <c:v>1.0125000000000006</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>4.0374999999999988</c:v>
+                  <c:v>1.0375000000000005</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>4.0624999999999991</c:v>
+                  <c:v>1.0625000000000004</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>4.0874999999999995</c:v>
+                  <c:v>1.0875000000000004</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>4.1124999999999998</c:v>
+                  <c:v>1.1125000000000003</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>4.1375000000000002</c:v>
+                  <c:v>1.1375000000000002</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>4.1625000000000005</c:v>
+                  <c:v>1.1625000000000001</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>4.1875000000000009</c:v>
+                  <c:v>1.1875</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>4.2125000000000012</c:v>
+                  <c:v>1.2124999999999999</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>4.2375000000000016</c:v>
+                  <c:v>1.2374999999999998</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>4.262500000000002</c:v>
+                  <c:v>1.2624999999999997</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>4.2875000000000023</c:v>
+                  <c:v>1.2874999999999996</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>4.3125000000000027</c:v>
+                  <c:v>1.3124999999999996</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>4.337500000000003</c:v>
+                  <c:v>1.3374999999999995</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>4.3625000000000034</c:v>
+                  <c:v>1.3624999999999994</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>4.3875000000000037</c:v>
+                  <c:v>1.3874999999999993</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>4.4125000000000041</c:v>
+                  <c:v>1.4124999999999992</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>4.4375000000000044</c:v>
+                  <c:v>1.4374999999999991</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>4.4625000000000048</c:v>
+                  <c:v>1.462499999999999</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>4.4875000000000052</c:v>
+                  <c:v>1.4874999999999989</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>4.5125000000000055</c:v>
+                  <c:v>1.5124999999999988</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>4.5375000000000059</c:v>
+                  <c:v>1.5374999999999988</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>4.5625000000000062</c:v>
+                  <c:v>1.5624999999999987</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>4.5875000000000066</c:v>
+                  <c:v>1.5874999999999986</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>4.6125000000000069</c:v>
+                  <c:v>1.6124999999999985</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>4.6375000000000073</c:v>
+                  <c:v>1.6374999999999984</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>4.6625000000000076</c:v>
+                  <c:v>1.6624999999999983</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>4.687500000000008</c:v>
+                  <c:v>1.6874999999999982</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>4.7125000000000083</c:v>
+                  <c:v>1.7124999999999981</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>4.7375000000000087</c:v>
+                  <c:v>1.737499999999998</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>4.7625000000000091</c:v>
+                  <c:v>1.762499999999998</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>4.7870000000000088</c:v>
+                  <c:v>1.7869999999999979</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>4.8105000000000091</c:v>
+                  <c:v>1.810499999999998</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>4.8330000000000091</c:v>
+                  <c:v>1.832999999999998</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>4.8545000000000087</c:v>
+                  <c:v>1.854499999999998</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>4.8750000000000089</c:v>
+                  <c:v>1.874999999999998</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>4.8945000000000087</c:v>
+                  <c:v>1.8944999999999981</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>4.9130000000000091</c:v>
+                  <c:v>1.912999999999998</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>4.9305000000000092</c:v>
+                  <c:v>1.9304999999999981</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>4.9470000000000089</c:v>
+                  <c:v>1.9469999999999981</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>4.9625000000000092</c:v>
+                  <c:v>1.9624999999999981</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>4.9770000000000092</c:v>
+                  <c:v>1.9769999999999981</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>4.9905000000000088</c:v>
+                  <c:v>1.9904999999999982</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>5.003000000000009</c:v>
+                  <c:v>2.0029999999999983</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>5.0145000000000088</c:v>
+                  <c:v>2.0144999999999982</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>5.0250000000000092</c:v>
+                  <c:v>2.0249999999999981</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>5.0345000000000093</c:v>
+                  <c:v>2.0344999999999982</c:v>
                 </c:pt>
                 <c:pt idx="96">
-                  <c:v>5.043000000000009</c:v>
+                  <c:v>2.0429999999999984</c:v>
                 </c:pt>
                 <c:pt idx="97">
-                  <c:v>5.0505000000000093</c:v>
+                  <c:v>2.0504999999999982</c:v>
                 </c:pt>
                 <c:pt idx="98">
-                  <c:v>5.0570000000000093</c:v>
+                  <c:v>2.0569999999999982</c:v>
                 </c:pt>
                 <c:pt idx="99">
-                  <c:v>5.0625000000000089</c:v>
+                  <c:v>2.0624999999999982</c:v>
                 </c:pt>
                 <c:pt idx="100">
-                  <c:v>5.0670000000000091</c:v>
+                  <c:v>2.0669999999999984</c:v>
                 </c:pt>
                 <c:pt idx="101">
-                  <c:v>5.0705000000000089</c:v>
+                  <c:v>2.0704999999999982</c:v>
                 </c:pt>
                 <c:pt idx="102">
-                  <c:v>5.0730000000000093</c:v>
+                  <c:v>2.0729999999999982</c:v>
                 </c:pt>
                 <c:pt idx="103">
-                  <c:v>5.0745000000000093</c:v>
+                  <c:v>2.0744999999999982</c:v>
                 </c:pt>
                 <c:pt idx="104">
-                  <c:v>5.0750000000000091</c:v>
+                  <c:v>2.0749999999999984</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5675,7 +5675,7 @@
         <v>0</v>
       </c>
       <c r="D2">
-        <v>3.1</v>
+        <v>0.1</v>
       </c>
       <c r="E2">
         <f>IF(A2&gt;0,A2*C2*100,0)</f>
@@ -5702,7 +5702,7 @@
       </c>
       <c r="D3">
         <f>(D2+(C2+0.5*A2)/1000)</f>
-        <v>3.1005000000000003</v>
+        <v>0.10050000000000001</v>
       </c>
       <c r="E3">
         <f t="shared" ref="E3:E86" si="1">IF(A3&gt;0,A3*C3*100,0)</f>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="D4">
         <f t="shared" ref="D4:D67" si="3">(D3+(C3+0.5*A3)/1000)</f>
-        <v>3.1020000000000003</v>
+        <v>0.10200000000000001</v>
       </c>
       <c r="E4">
         <f t="shared" si="1"/>
@@ -5750,7 +5750,7 @@
       </c>
       <c r="D5">
         <f t="shared" si="3"/>
-        <v>3.1045000000000003</v>
+        <v>0.10450000000000001</v>
       </c>
       <c r="E5">
         <f t="shared" si="1"/>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="D6">
         <f t="shared" si="3"/>
-        <v>3.1080000000000001</v>
+        <v>0.10800000000000001</v>
       </c>
       <c r="E6">
         <f t="shared" si="1"/>
@@ -5798,7 +5798,7 @@
       </c>
       <c r="D7">
         <f t="shared" si="3"/>
-        <v>3.1125000000000003</v>
+        <v>0.11250000000000002</v>
       </c>
       <c r="E7">
         <f t="shared" si="1"/>
@@ -5822,7 +5822,7 @@
       </c>
       <c r="D8">
         <f t="shared" si="3"/>
-        <v>3.1180000000000003</v>
+        <v>0.11800000000000002</v>
       </c>
       <c r="E8">
         <f t="shared" si="1"/>
@@ -5846,7 +5846,7 @@
       </c>
       <c r="D9">
         <f t="shared" si="3"/>
-        <v>3.1245000000000003</v>
+        <v>0.12450000000000003</v>
       </c>
       <c r="E9">
         <f t="shared" si="1"/>
@@ -5870,7 +5870,7 @@
       </c>
       <c r="D10">
         <f t="shared" si="3"/>
-        <v>3.1320000000000001</v>
+        <v>0.13200000000000003</v>
       </c>
       <c r="E10">
         <f t="shared" si="1"/>
@@ -5894,7 +5894,7 @@
       </c>
       <c r="D11">
         <f t="shared" si="3"/>
-        <v>3.1405000000000003</v>
+        <v>0.14050000000000004</v>
       </c>
       <c r="E11">
         <f t="shared" si="1"/>
@@ -5918,7 +5918,7 @@
       </c>
       <c r="D12">
         <f t="shared" si="3"/>
-        <v>3.1500000000000004</v>
+        <v>0.15000000000000005</v>
       </c>
       <c r="E12">
         <f t="shared" si="1"/>
@@ -5942,7 +5942,7 @@
       </c>
       <c r="D13">
         <f t="shared" si="3"/>
-        <v>3.1605000000000003</v>
+        <v>0.16050000000000006</v>
       </c>
       <c r="E13">
         <f t="shared" si="1"/>
@@ -5966,7 +5966,7 @@
       </c>
       <c r="D14">
         <f t="shared" si="3"/>
-        <v>3.1720000000000002</v>
+        <v>0.17200000000000007</v>
       </c>
       <c r="E14">
         <f t="shared" si="1"/>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="D15">
         <f t="shared" si="3"/>
-        <v>3.1845000000000003</v>
+        <v>0.18450000000000008</v>
       </c>
       <c r="E15">
         <f t="shared" si="1"/>
@@ -6014,7 +6014,7 @@
       </c>
       <c r="D16">
         <f t="shared" si="3"/>
-        <v>3.1980000000000004</v>
+        <v>0.19800000000000009</v>
       </c>
       <c r="E16">
         <f t="shared" si="1"/>
@@ -6038,7 +6038,7 @@
       </c>
       <c r="D17">
         <f t="shared" si="3"/>
-        <v>3.2125000000000004</v>
+        <v>0.21250000000000011</v>
       </c>
       <c r="E17">
         <f t="shared" si="1"/>
@@ -6062,7 +6062,7 @@
       </c>
       <c r="D18">
         <f t="shared" si="3"/>
-        <v>3.2280000000000002</v>
+        <v>0.22800000000000009</v>
       </c>
       <c r="E18">
         <f t="shared" si="1"/>
@@ -6086,7 +6086,7 @@
       </c>
       <c r="D19">
         <f t="shared" si="3"/>
-        <v>3.2445000000000004</v>
+        <v>0.24450000000000011</v>
       </c>
       <c r="E19">
         <f t="shared" si="1"/>
@@ -6110,7 +6110,7 @@
       </c>
       <c r="D20">
         <f t="shared" si="3"/>
-        <v>3.2620000000000005</v>
+        <v>0.26200000000000012</v>
       </c>
       <c r="E20">
         <f t="shared" si="1"/>
@@ -6134,7 +6134,7 @@
       </c>
       <c r="D21">
         <f t="shared" si="3"/>
-        <v>3.2805000000000004</v>
+        <v>0.28050000000000014</v>
       </c>
       <c r="E21">
         <f t="shared" si="1"/>
@@ -6158,7 +6158,7 @@
       </c>
       <c r="D22">
         <f t="shared" si="3"/>
-        <v>3.3000000000000003</v>
+        <v>0.30000000000000016</v>
       </c>
       <c r="E22">
         <f t="shared" si="1"/>
@@ -6182,7 +6182,7 @@
       </c>
       <c r="D23">
         <f t="shared" si="3"/>
-        <v>3.3205000000000005</v>
+        <v>0.32050000000000017</v>
       </c>
       <c r="E23">
         <f t="shared" si="1"/>
@@ -6206,7 +6206,7 @@
       </c>
       <c r="D24">
         <f t="shared" si="3"/>
-        <v>3.3420000000000005</v>
+        <v>0.34200000000000019</v>
       </c>
       <c r="E24">
         <f t="shared" si="1"/>
@@ -6230,7 +6230,7 @@
       </c>
       <c r="D25">
         <f t="shared" si="3"/>
-        <v>3.3645000000000005</v>
+        <v>0.36450000000000021</v>
       </c>
       <c r="E25">
         <f t="shared" si="1"/>
@@ -6254,7 +6254,7 @@
       </c>
       <c r="D26">
         <f t="shared" si="3"/>
-        <v>3.3880000000000003</v>
+        <v>0.38800000000000023</v>
       </c>
       <c r="E26">
         <f t="shared" si="1"/>
@@ -6281,7 +6281,7 @@
       </c>
       <c r="D27">
         <f t="shared" si="3"/>
-        <v>3.4125000000000005</v>
+        <v>0.41250000000000026</v>
       </c>
       <c r="E27">
         <f t="shared" si="1"/>
@@ -6305,7 +6305,7 @@
       </c>
       <c r="D28">
         <f t="shared" si="3"/>
-        <v>3.4375000000000004</v>
+        <v>0.43750000000000028</v>
       </c>
       <c r="E28">
         <f t="shared" si="1"/>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="D29">
         <f t="shared" si="3"/>
-        <v>3.4625000000000004</v>
+        <v>0.4625000000000003</v>
       </c>
       <c r="E29">
         <f t="shared" ref="E29:E45" si="5">IF(A29&gt;0,A29*C29*100,0)</f>
@@ -6353,7 +6353,7 @@
       </c>
       <c r="D30">
         <f t="shared" si="3"/>
-        <v>3.4875000000000003</v>
+        <v>0.48750000000000032</v>
       </c>
       <c r="E30">
         <f t="shared" si="5"/>
@@ -6377,7 +6377,7 @@
       </c>
       <c r="D31">
         <f t="shared" si="3"/>
-        <v>3.5125000000000002</v>
+        <v>0.51250000000000029</v>
       </c>
       <c r="E31">
         <f t="shared" si="5"/>
@@ -6401,7 +6401,7 @@
       </c>
       <c r="D32">
         <f t="shared" si="3"/>
-        <v>3.5375000000000001</v>
+        <v>0.53750000000000031</v>
       </c>
       <c r="E32">
         <f t="shared" si="5"/>
@@ -6425,7 +6425,7 @@
       </c>
       <c r="D33">
         <f t="shared" si="3"/>
-        <v>3.5625</v>
+        <v>0.56250000000000033</v>
       </c>
       <c r="E33">
         <f t="shared" si="5"/>
@@ -6449,7 +6449,7 @@
       </c>
       <c r="D34">
         <f t="shared" si="3"/>
-        <v>3.5874999999999999</v>
+        <v>0.58750000000000036</v>
       </c>
       <c r="E34">
         <f t="shared" si="5"/>
@@ -6473,7 +6473,7 @@
       </c>
       <c r="D35">
         <f t="shared" si="3"/>
-        <v>3.6124999999999998</v>
+        <v>0.61250000000000038</v>
       </c>
       <c r="E35">
         <f t="shared" si="5"/>
@@ -6497,7 +6497,7 @@
       </c>
       <c r="D36">
         <f t="shared" si="3"/>
-        <v>3.6374999999999997</v>
+        <v>0.6375000000000004</v>
       </c>
       <c r="E36">
         <f t="shared" si="5"/>
@@ -6521,7 +6521,7 @@
       </c>
       <c r="D37">
         <f t="shared" si="3"/>
-        <v>3.6624999999999996</v>
+        <v>0.66250000000000042</v>
       </c>
       <c r="E37">
         <f t="shared" si="5"/>
@@ -6545,7 +6545,7 @@
       </c>
       <c r="D38">
         <f t="shared" si="3"/>
-        <v>3.6874999999999996</v>
+        <v>0.68750000000000044</v>
       </c>
       <c r="E38">
         <f t="shared" si="5"/>
@@ -6569,7 +6569,7 @@
       </c>
       <c r="D39">
         <f t="shared" si="3"/>
-        <v>3.7124999999999995</v>
+        <v>0.71250000000000047</v>
       </c>
       <c r="E39">
         <f t="shared" si="5"/>
@@ -6593,7 +6593,7 @@
       </c>
       <c r="D40">
         <f t="shared" si="3"/>
-        <v>3.7374999999999994</v>
+        <v>0.73750000000000049</v>
       </c>
       <c r="E40">
         <f t="shared" si="5"/>
@@ -6617,7 +6617,7 @@
       </c>
       <c r="D41">
         <f t="shared" si="3"/>
-        <v>3.7624999999999993</v>
+        <v>0.76250000000000051</v>
       </c>
       <c r="E41">
         <f t="shared" si="5"/>
@@ -6641,7 +6641,7 @@
       </c>
       <c r="D42">
         <f t="shared" si="3"/>
-        <v>3.7874999999999992</v>
+        <v>0.78750000000000053</v>
       </c>
       <c r="E42">
         <f t="shared" si="5"/>
@@ -6665,7 +6665,7 @@
       </c>
       <c r="D43">
         <f t="shared" si="3"/>
-        <v>3.8124999999999991</v>
+        <v>0.81250000000000056</v>
       </c>
       <c r="E43">
         <f t="shared" si="5"/>
@@ -6689,7 +6689,7 @@
       </c>
       <c r="D44">
         <f t="shared" si="3"/>
-        <v>3.837499999999999</v>
+        <v>0.83750000000000058</v>
       </c>
       <c r="E44">
         <f t="shared" si="5"/>
@@ -6713,7 +6713,7 @@
       </c>
       <c r="D45">
         <f t="shared" si="3"/>
-        <v>3.8624999999999989</v>
+        <v>0.8625000000000006</v>
       </c>
       <c r="E45">
         <f t="shared" si="5"/>
@@ -6737,7 +6737,7 @@
       </c>
       <c r="D46">
         <f t="shared" si="3"/>
-        <v>3.8874999999999988</v>
+        <v>0.88750000000000062</v>
       </c>
       <c r="E46">
         <f t="shared" ref="E46:E80" si="8">IF(A46&gt;0,A46*C46*100,0)</f>
@@ -6761,7 +6761,7 @@
       </c>
       <c r="D47">
         <f t="shared" si="3"/>
-        <v>3.9124999999999988</v>
+        <v>0.91250000000000064</v>
       </c>
       <c r="E47">
         <f t="shared" si="8"/>
@@ -6785,7 +6785,7 @@
       </c>
       <c r="D48">
         <f t="shared" si="3"/>
-        <v>3.9374999999999987</v>
+        <v>0.93750000000000067</v>
       </c>
       <c r="E48">
         <f t="shared" si="8"/>
@@ -6809,7 +6809,7 @@
       </c>
       <c r="D49">
         <f t="shared" si="3"/>
-        <v>3.9624999999999986</v>
+        <v>0.96250000000000069</v>
       </c>
       <c r="E49">
         <f t="shared" si="8"/>
@@ -6833,7 +6833,7 @@
       </c>
       <c r="D50">
         <f t="shared" si="3"/>
-        <v>3.9874999999999985</v>
+        <v>0.98750000000000071</v>
       </c>
       <c r="E50">
         <f t="shared" si="8"/>
@@ -6857,7 +6857,7 @@
       </c>
       <c r="D51">
         <f t="shared" si="3"/>
-        <v>4.0124999999999984</v>
+        <v>1.0125000000000006</v>
       </c>
       <c r="E51">
         <f t="shared" si="8"/>
@@ -6881,7 +6881,7 @@
       </c>
       <c r="D52">
         <f t="shared" si="3"/>
-        <v>4.0374999999999988</v>
+        <v>1.0375000000000005</v>
       </c>
       <c r="E52">
         <f t="shared" si="8"/>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="D53">
         <f t="shared" si="3"/>
-        <v>4.0624999999999991</v>
+        <v>1.0625000000000004</v>
       </c>
       <c r="E53">
         <f t="shared" si="8"/>
@@ -6929,7 +6929,7 @@
       </c>
       <c r="D54">
         <f t="shared" si="3"/>
-        <v>4.0874999999999995</v>
+        <v>1.0875000000000004</v>
       </c>
       <c r="E54">
         <f t="shared" si="8"/>
@@ -6953,7 +6953,7 @@
       </c>
       <c r="D55">
         <f t="shared" si="3"/>
-        <v>4.1124999999999998</v>
+        <v>1.1125000000000003</v>
       </c>
       <c r="E55">
         <f t="shared" si="8"/>
@@ -6977,7 +6977,7 @@
       </c>
       <c r="D56">
         <f t="shared" si="3"/>
-        <v>4.1375000000000002</v>
+        <v>1.1375000000000002</v>
       </c>
       <c r="E56">
         <f t="shared" si="8"/>
@@ -7001,7 +7001,7 @@
       </c>
       <c r="D57">
         <f t="shared" si="3"/>
-        <v>4.1625000000000005</v>
+        <v>1.1625000000000001</v>
       </c>
       <c r="E57">
         <f t="shared" si="8"/>
@@ -7025,7 +7025,7 @@
       </c>
       <c r="D58">
         <f t="shared" si="3"/>
-        <v>4.1875000000000009</v>
+        <v>1.1875</v>
       </c>
       <c r="E58">
         <f t="shared" si="8"/>
@@ -7049,7 +7049,7 @@
       </c>
       <c r="D59">
         <f t="shared" si="3"/>
-        <v>4.2125000000000012</v>
+        <v>1.2124999999999999</v>
       </c>
       <c r="E59">
         <f t="shared" si="8"/>
@@ -7073,7 +7073,7 @@
       </c>
       <c r="D60">
         <f t="shared" si="3"/>
-        <v>4.2375000000000016</v>
+        <v>1.2374999999999998</v>
       </c>
       <c r="E60">
         <f t="shared" si="8"/>
@@ -7097,7 +7097,7 @@
       </c>
       <c r="D61">
         <f t="shared" si="3"/>
-        <v>4.262500000000002</v>
+        <v>1.2624999999999997</v>
       </c>
       <c r="E61">
         <f t="shared" si="8"/>
@@ -7121,7 +7121,7 @@
       </c>
       <c r="D62">
         <f t="shared" si="3"/>
-        <v>4.2875000000000023</v>
+        <v>1.2874999999999996</v>
       </c>
       <c r="E62">
         <f t="shared" si="8"/>
@@ -7145,7 +7145,7 @@
       </c>
       <c r="D63">
         <f t="shared" si="3"/>
-        <v>4.3125000000000027</v>
+        <v>1.3124999999999996</v>
       </c>
       <c r="E63">
         <f t="shared" si="8"/>
@@ -7169,7 +7169,7 @@
       </c>
       <c r="D64">
         <f t="shared" si="3"/>
-        <v>4.337500000000003</v>
+        <v>1.3374999999999995</v>
       </c>
       <c r="E64">
         <f t="shared" si="8"/>
@@ -7193,7 +7193,7 @@
       </c>
       <c r="D65">
         <f t="shared" si="3"/>
-        <v>4.3625000000000034</v>
+        <v>1.3624999999999994</v>
       </c>
       <c r="E65">
         <f t="shared" si="8"/>
@@ -7217,7 +7217,7 @@
       </c>
       <c r="D66">
         <f t="shared" si="3"/>
-        <v>4.3875000000000037</v>
+        <v>1.3874999999999993</v>
       </c>
       <c r="E66">
         <f t="shared" ref="E66:E68" si="11">IF(A66&gt;0,A66*C66*100,0)</f>
@@ -7241,7 +7241,7 @@
       </c>
       <c r="D67">
         <f t="shared" si="3"/>
-        <v>4.4125000000000041</v>
+        <v>1.4124999999999992</v>
       </c>
       <c r="E67">
         <f t="shared" si="11"/>
@@ -7265,7 +7265,7 @@
       </c>
       <c r="D68">
         <f t="shared" ref="D68:D106" si="13">(D67+(C67+0.5*A67)/1000)</f>
-        <v>4.4375000000000044</v>
+        <v>1.4374999999999991</v>
       </c>
       <c r="E68">
         <f t="shared" si="11"/>
@@ -7289,7 +7289,7 @@
       </c>
       <c r="D69">
         <f t="shared" si="13"/>
-        <v>4.4625000000000048</v>
+        <v>1.462499999999999</v>
       </c>
       <c r="E69">
         <f t="shared" ref="E69:E71" si="15">IF(A69&gt;0,A69*C69*100,0)</f>
@@ -7313,7 +7313,7 @@
       </c>
       <c r="D70">
         <f t="shared" si="13"/>
-        <v>4.4875000000000052</v>
+        <v>1.4874999999999989</v>
       </c>
       <c r="E70">
         <f t="shared" si="15"/>
@@ -7337,7 +7337,7 @@
       </c>
       <c r="D71">
         <f t="shared" si="13"/>
-        <v>4.5125000000000055</v>
+        <v>1.5124999999999988</v>
       </c>
       <c r="E71">
         <f t="shared" si="15"/>
@@ -7361,7 +7361,7 @@
       </c>
       <c r="D72">
         <f t="shared" si="13"/>
-        <v>4.5375000000000059</v>
+        <v>1.5374999999999988</v>
       </c>
       <c r="E72">
         <f t="shared" si="8"/>
@@ -7385,7 +7385,7 @@
       </c>
       <c r="D73">
         <f t="shared" si="13"/>
-        <v>4.5625000000000062</v>
+        <v>1.5624999999999987</v>
       </c>
       <c r="E73">
         <f t="shared" si="8"/>
@@ -7409,7 +7409,7 @@
       </c>
       <c r="D74">
         <f t="shared" si="13"/>
-        <v>4.5875000000000066</v>
+        <v>1.5874999999999986</v>
       </c>
       <c r="E74">
         <f t="shared" si="8"/>
@@ -7436,7 +7436,7 @@
       </c>
       <c r="D75">
         <f t="shared" si="13"/>
-        <v>4.6125000000000069</v>
+        <v>1.6124999999999985</v>
       </c>
       <c r="E75">
         <f t="shared" si="8"/>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="D76">
         <f t="shared" si="13"/>
-        <v>4.6375000000000073</v>
+        <v>1.6374999999999984</v>
       </c>
       <c r="E76">
         <f t="shared" si="8"/>
@@ -7484,7 +7484,7 @@
       </c>
       <c r="D77">
         <f t="shared" si="13"/>
-        <v>4.6625000000000076</v>
+        <v>1.6624999999999983</v>
       </c>
       <c r="E77">
         <f t="shared" si="8"/>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D78">
         <f t="shared" si="13"/>
-        <v>4.687500000000008</v>
+        <v>1.6874999999999982</v>
       </c>
       <c r="E78">
         <f t="shared" si="8"/>
@@ -7532,7 +7532,7 @@
       </c>
       <c r="D79">
         <f t="shared" si="13"/>
-        <v>4.7125000000000083</v>
+        <v>1.7124999999999981</v>
       </c>
       <c r="E79">
         <f t="shared" si="8"/>
@@ -7556,7 +7556,7 @@
       </c>
       <c r="D80">
         <f t="shared" si="13"/>
-        <v>4.7375000000000087</v>
+        <v>1.737499999999998</v>
       </c>
       <c r="E80">
         <f t="shared" si="8"/>
@@ -7580,7 +7580,7 @@
       </c>
       <c r="D81">
         <f t="shared" si="13"/>
-        <v>4.7625000000000091</v>
+        <v>1.762499999999998</v>
       </c>
       <c r="E81">
         <f t="shared" si="1"/>
@@ -7604,7 +7604,7 @@
       </c>
       <c r="D82">
         <f t="shared" si="13"/>
-        <v>4.7870000000000088</v>
+        <v>1.7869999999999979</v>
       </c>
       <c r="E82">
         <f t="shared" si="1"/>
@@ -7628,7 +7628,7 @@
       </c>
       <c r="D83">
         <f t="shared" si="13"/>
-        <v>4.8105000000000091</v>
+        <v>1.810499999999998</v>
       </c>
       <c r="E83">
         <f t="shared" si="1"/>
@@ -7652,7 +7652,7 @@
       </c>
       <c r="D84">
         <f t="shared" si="13"/>
-        <v>4.8330000000000091</v>
+        <v>1.832999999999998</v>
       </c>
       <c r="E84">
         <f t="shared" si="1"/>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="D85">
         <f t="shared" si="13"/>
-        <v>4.8545000000000087</v>
+        <v>1.854499999999998</v>
       </c>
       <c r="E85">
         <f t="shared" si="1"/>
@@ -7700,7 +7700,7 @@
       </c>
       <c r="D86">
         <f t="shared" si="13"/>
-        <v>4.8750000000000089</v>
+        <v>1.874999999999998</v>
       </c>
       <c r="E86">
         <f t="shared" si="1"/>
@@ -7724,7 +7724,7 @@
       </c>
       <c r="D87">
         <f t="shared" si="13"/>
-        <v>4.8945000000000087</v>
+        <v>1.8944999999999981</v>
       </c>
       <c r="E87">
         <f t="shared" ref="E87:E91" si="18">IF(A87&gt;0,A87*C87*100,0)</f>
@@ -7748,7 +7748,7 @@
       </c>
       <c r="D88">
         <f t="shared" si="13"/>
-        <v>4.9130000000000091</v>
+        <v>1.912999999999998</v>
       </c>
       <c r="E88">
         <f t="shared" si="18"/>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D89">
         <f t="shared" si="13"/>
-        <v>4.9305000000000092</v>
+        <v>1.9304999999999981</v>
       </c>
       <c r="E89">
         <f t="shared" si="18"/>
@@ -7796,7 +7796,7 @@
       </c>
       <c r="D90">
         <f t="shared" si="13"/>
-        <v>4.9470000000000089</v>
+        <v>1.9469999999999981</v>
       </c>
       <c r="E90">
         <f t="shared" si="18"/>
@@ -7820,7 +7820,7 @@
       </c>
       <c r="D91">
         <f t="shared" si="13"/>
-        <v>4.9625000000000092</v>
+        <v>1.9624999999999981</v>
       </c>
       <c r="E91">
         <f t="shared" si="18"/>
@@ -7844,7 +7844,7 @@
       </c>
       <c r="D92">
         <f t="shared" si="13"/>
-        <v>4.9770000000000092</v>
+        <v>1.9769999999999981</v>
       </c>
       <c r="E92">
         <f t="shared" ref="E92:E103" si="20">IF(A92&gt;0,A92*C92*100,0)</f>
@@ -7868,7 +7868,7 @@
       </c>
       <c r="D93">
         <f t="shared" si="13"/>
-        <v>4.9905000000000088</v>
+        <v>1.9904999999999982</v>
       </c>
       <c r="E93">
         <f t="shared" si="20"/>
@@ -7892,7 +7892,7 @@
       </c>
       <c r="D94">
         <f t="shared" si="13"/>
-        <v>5.003000000000009</v>
+        <v>2.0029999999999983</v>
       </c>
       <c r="E94">
         <f t="shared" si="20"/>
@@ -7916,7 +7916,7 @@
       </c>
       <c r="D95">
         <f t="shared" si="13"/>
-        <v>5.0145000000000088</v>
+        <v>2.0144999999999982</v>
       </c>
       <c r="E95">
         <f t="shared" si="20"/>
@@ -7940,7 +7940,7 @@
       </c>
       <c r="D96">
         <f t="shared" si="13"/>
-        <v>5.0250000000000092</v>
+        <v>2.0249999999999981</v>
       </c>
       <c r="E96">
         <f t="shared" si="20"/>
@@ -7964,7 +7964,7 @@
       </c>
       <c r="D97">
         <f t="shared" si="13"/>
-        <v>5.0345000000000093</v>
+        <v>2.0344999999999982</v>
       </c>
       <c r="E97">
         <f t="shared" si="20"/>
@@ -7988,7 +7988,7 @@
       </c>
       <c r="D98">
         <f t="shared" si="13"/>
-        <v>5.043000000000009</v>
+        <v>2.0429999999999984</v>
       </c>
       <c r="E98">
         <f t="shared" si="20"/>
@@ -8012,7 +8012,7 @@
       </c>
       <c r="D99">
         <f t="shared" si="13"/>
-        <v>5.0505000000000093</v>
+        <v>2.0504999999999982</v>
       </c>
       <c r="E99">
         <f t="shared" si="20"/>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D100">
         <f t="shared" si="13"/>
-        <v>5.0570000000000093</v>
+        <v>2.0569999999999982</v>
       </c>
       <c r="E100">
         <f t="shared" si="20"/>
@@ -8060,7 +8060,7 @@
       </c>
       <c r="D101">
         <f t="shared" si="13"/>
-        <v>5.0625000000000089</v>
+        <v>2.0624999999999982</v>
       </c>
       <c r="E101">
         <f t="shared" si="20"/>
@@ -8084,7 +8084,7 @@
       </c>
       <c r="D102">
         <f t="shared" si="13"/>
-        <v>5.0670000000000091</v>
+        <v>2.0669999999999984</v>
       </c>
       <c r="E102">
         <f t="shared" si="20"/>
@@ -8108,7 +8108,7 @@
       </c>
       <c r="D103">
         <f t="shared" si="13"/>
-        <v>5.0705000000000089</v>
+        <v>2.0704999999999982</v>
       </c>
       <c r="E103">
         <f t="shared" si="20"/>
@@ -8132,7 +8132,7 @@
       </c>
       <c r="D104">
         <f t="shared" si="13"/>
-        <v>5.0730000000000093</v>
+        <v>2.0729999999999982</v>
       </c>
       <c r="E104">
         <f t="shared" ref="E104:E106" si="22">IF(A104&gt;0,A104*C104*100,0)</f>
@@ -8156,7 +8156,7 @@
       </c>
       <c r="D105">
         <f t="shared" si="13"/>
-        <v>5.0745000000000093</v>
+        <v>2.0744999999999982</v>
       </c>
       <c r="E105">
         <f t="shared" si="22"/>
@@ -8180,7 +8180,7 @@
       </c>
       <c r="D106">
         <f t="shared" si="13"/>
-        <v>5.0750000000000091</v>
+        <v>2.0749999999999984</v>
       </c>
       <c r="E106">
         <f t="shared" si="22"/>

</xml_diff>